<commit_message>
Rename Akshay Antony to Akshay A in the participants workbook
Matches the name now used in the Google Sheet's brackets, and rebuilds
data/snapshot.json.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJbwidL2Cpt5zaaQmJxQ9m
</commit_message>
<xml_diff>
--- a/data/Vonnue_Cup_Participants.xlsx
+++ b/data/Vonnue_Cup_Participants.xlsx
@@ -6934,7 +6934,7 @@
       </c>
       <c r="F127" s="10" t="inlineStr">
         <is>
-          <t>Akshay Antony</t>
+          <t>Akshay A</t>
         </is>
       </c>
       <c r="G127" s="10" t="n"/>
@@ -14573,7 +14573,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Akshay Antony</t>
+          <t>Akshay A</t>
         </is>
       </c>
       <c r="D6" s="6" t="n"/>

</xml_diff>

<commit_message>
Sync new badminton draw and full player names from the Google Sheet
Badminton: 12 entries per event (2 per team), teammates in opposite halves, new order of play
for Sun 01 Nov ending 18:37. Participants: new badminton lists and full names across all sports.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XgUQLqsKTbyKtnK2HPdyHV
</commit_message>
<xml_diff>
--- a/data/Vonnue_Cup_Participants.xlsx
+++ b/data/Vonnue_Cup_Participants.xlsx
@@ -295,7 +295,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AllEntries" displayName="AllEntries" ref="A1:H156" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AllEntries" displayName="AllEntries" ref="A1:H158" headerRowCount="1">
   <tableColumns count="8">
     <tableColumn id="1" name="#"/>
     <tableColumn id="2" name="Team"/>
@@ -535,6 +535,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1" s="15">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -604,27 +605,27 @@
         </is>
       </c>
       <c r="D5" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,D$4,'All Entries'!$C$2:$C$156,$A5,'All Entries'!$E$2:$E$156,$B5,'All Entries'!$D$2:$D$156,$C5)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,D$4,'All Entries'!$C$2:$C$158,$A5,'All Entries'!$E$2:$E$158,$B5,'All Entries'!$D$2:$D$158,$C5)</f>
         <v/>
       </c>
       <c r="E5" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,E$4,'All Entries'!$C$2:$C$156,$A5,'All Entries'!$E$2:$E$156,$B5,'All Entries'!$D$2:$D$156,$C5)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,E$4,'All Entries'!$C$2:$C$158,$A5,'All Entries'!$E$2:$E$158,$B5,'All Entries'!$D$2:$D$158,$C5)</f>
         <v/>
       </c>
       <c r="F5" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,F$4,'All Entries'!$C$2:$C$156,$A5,'All Entries'!$E$2:$E$156,$B5,'All Entries'!$D$2:$D$156,$C5)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,F$4,'All Entries'!$C$2:$C$158,$A5,'All Entries'!$E$2:$E$158,$B5,'All Entries'!$D$2:$D$158,$C5)</f>
         <v/>
       </c>
       <c r="G5" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,G$4,'All Entries'!$C$2:$C$156,$A5,'All Entries'!$E$2:$E$156,$B5,'All Entries'!$D$2:$D$156,$C5)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,G$4,'All Entries'!$C$2:$C$158,$A5,'All Entries'!$E$2:$E$158,$B5,'All Entries'!$D$2:$D$158,$C5)</f>
         <v/>
       </c>
       <c r="H5" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,H$4,'All Entries'!$C$2:$C$156,$A5,'All Entries'!$E$2:$E$156,$B5,'All Entries'!$D$2:$D$156,$C5)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,H$4,'All Entries'!$C$2:$C$158,$A5,'All Entries'!$E$2:$E$158,$B5,'All Entries'!$D$2:$D$158,$C5)</f>
         <v/>
       </c>
       <c r="I5" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,I$4,'All Entries'!$C$2:$C$156,$A5,'All Entries'!$E$2:$E$156,$B5,'All Entries'!$D$2:$D$156,$C5)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,I$4,'All Entries'!$C$2:$C$158,$A5,'All Entries'!$E$2:$E$158,$B5,'All Entries'!$D$2:$D$158,$C5)</f>
         <v/>
       </c>
       <c r="J5" s="11">
@@ -649,27 +650,27 @@
         </is>
       </c>
       <c r="D6" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,D$4,'All Entries'!$C$2:$C$156,$A6,'All Entries'!$E$2:$E$156,$B6,'All Entries'!$D$2:$D$156,$C6)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,D$4,'All Entries'!$C$2:$C$158,$A6,'All Entries'!$E$2:$E$158,$B6,'All Entries'!$D$2:$D$158,$C6)</f>
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,E$4,'All Entries'!$C$2:$C$156,$A6,'All Entries'!$E$2:$E$156,$B6,'All Entries'!$D$2:$D$156,$C6)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,E$4,'All Entries'!$C$2:$C$158,$A6,'All Entries'!$E$2:$E$158,$B6,'All Entries'!$D$2:$D$158,$C6)</f>
         <v/>
       </c>
       <c r="F6" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,F$4,'All Entries'!$C$2:$C$156,$A6,'All Entries'!$E$2:$E$156,$B6,'All Entries'!$D$2:$D$156,$C6)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,F$4,'All Entries'!$C$2:$C$158,$A6,'All Entries'!$E$2:$E$158,$B6,'All Entries'!$D$2:$D$158,$C6)</f>
         <v/>
       </c>
       <c r="G6" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,G$4,'All Entries'!$C$2:$C$156,$A6,'All Entries'!$E$2:$E$156,$B6,'All Entries'!$D$2:$D$156,$C6)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,G$4,'All Entries'!$C$2:$C$158,$A6,'All Entries'!$E$2:$E$158,$B6,'All Entries'!$D$2:$D$158,$C6)</f>
         <v/>
       </c>
       <c r="H6" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,H$4,'All Entries'!$C$2:$C$156,$A6,'All Entries'!$E$2:$E$156,$B6,'All Entries'!$D$2:$D$156,$C6)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,H$4,'All Entries'!$C$2:$C$158,$A6,'All Entries'!$E$2:$E$158,$B6,'All Entries'!$D$2:$D$158,$C6)</f>
         <v/>
       </c>
       <c r="I6" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,I$4,'All Entries'!$C$2:$C$156,$A6,'All Entries'!$E$2:$E$156,$B6,'All Entries'!$D$2:$D$156,$C6)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,I$4,'All Entries'!$C$2:$C$158,$A6,'All Entries'!$E$2:$E$158,$B6,'All Entries'!$D$2:$D$158,$C6)</f>
         <v/>
       </c>
       <c r="J6" s="11">
@@ -694,27 +695,27 @@
         </is>
       </c>
       <c r="D7" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,D$4,'All Entries'!$C$2:$C$156,$A7,'All Entries'!$E$2:$E$156,$B7,'All Entries'!$D$2:$D$156,$C7)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,D$4,'All Entries'!$C$2:$C$158,$A7,'All Entries'!$E$2:$E$158,$B7,'All Entries'!$D$2:$D$158,$C7)</f>
         <v/>
       </c>
       <c r="E7" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,E$4,'All Entries'!$C$2:$C$156,$A7,'All Entries'!$E$2:$E$156,$B7,'All Entries'!$D$2:$D$156,$C7)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,E$4,'All Entries'!$C$2:$C$158,$A7,'All Entries'!$E$2:$E$158,$B7,'All Entries'!$D$2:$D$158,$C7)</f>
         <v/>
       </c>
       <c r="F7" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,F$4,'All Entries'!$C$2:$C$156,$A7,'All Entries'!$E$2:$E$156,$B7,'All Entries'!$D$2:$D$156,$C7)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,F$4,'All Entries'!$C$2:$C$158,$A7,'All Entries'!$E$2:$E$158,$B7,'All Entries'!$D$2:$D$158,$C7)</f>
         <v/>
       </c>
       <c r="G7" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,G$4,'All Entries'!$C$2:$C$156,$A7,'All Entries'!$E$2:$E$156,$B7,'All Entries'!$D$2:$D$156,$C7)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,G$4,'All Entries'!$C$2:$C$158,$A7,'All Entries'!$E$2:$E$158,$B7,'All Entries'!$D$2:$D$158,$C7)</f>
         <v/>
       </c>
       <c r="H7" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,H$4,'All Entries'!$C$2:$C$156,$A7,'All Entries'!$E$2:$E$156,$B7,'All Entries'!$D$2:$D$156,$C7)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,H$4,'All Entries'!$C$2:$C$158,$A7,'All Entries'!$E$2:$E$158,$B7,'All Entries'!$D$2:$D$158,$C7)</f>
         <v/>
       </c>
       <c r="I7" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,I$4,'All Entries'!$C$2:$C$156,$A7,'All Entries'!$E$2:$E$156,$B7,'All Entries'!$D$2:$D$156,$C7)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,I$4,'All Entries'!$C$2:$C$158,$A7,'All Entries'!$E$2:$E$158,$B7,'All Entries'!$D$2:$D$158,$C7)</f>
         <v/>
       </c>
       <c r="J7" s="11">
@@ -739,27 +740,27 @@
         </is>
       </c>
       <c r="D8" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,D$4,'All Entries'!$C$2:$C$156,$A8,'All Entries'!$E$2:$E$156,$B8,'All Entries'!$D$2:$D$156,$C8)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,D$4,'All Entries'!$C$2:$C$158,$A8,'All Entries'!$E$2:$E$158,$B8,'All Entries'!$D$2:$D$158,$C8)</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,E$4,'All Entries'!$C$2:$C$156,$A8,'All Entries'!$E$2:$E$156,$B8,'All Entries'!$D$2:$D$156,$C8)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,E$4,'All Entries'!$C$2:$C$158,$A8,'All Entries'!$E$2:$E$158,$B8,'All Entries'!$D$2:$D$158,$C8)</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,F$4,'All Entries'!$C$2:$C$156,$A8,'All Entries'!$E$2:$E$156,$B8,'All Entries'!$D$2:$D$156,$C8)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,F$4,'All Entries'!$C$2:$C$158,$A8,'All Entries'!$E$2:$E$158,$B8,'All Entries'!$D$2:$D$158,$C8)</f>
         <v/>
       </c>
       <c r="G8" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,G$4,'All Entries'!$C$2:$C$156,$A8,'All Entries'!$E$2:$E$156,$B8,'All Entries'!$D$2:$D$156,$C8)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,G$4,'All Entries'!$C$2:$C$158,$A8,'All Entries'!$E$2:$E$158,$B8,'All Entries'!$D$2:$D$158,$C8)</f>
         <v/>
       </c>
       <c r="H8" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,H$4,'All Entries'!$C$2:$C$156,$A8,'All Entries'!$E$2:$E$156,$B8,'All Entries'!$D$2:$D$156,$C8)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,H$4,'All Entries'!$C$2:$C$158,$A8,'All Entries'!$E$2:$E$158,$B8,'All Entries'!$D$2:$D$158,$C8)</f>
         <v/>
       </c>
       <c r="I8" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,I$4,'All Entries'!$C$2:$C$156,$A8,'All Entries'!$E$2:$E$156,$B8,'All Entries'!$D$2:$D$156,$C8)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,I$4,'All Entries'!$C$2:$C$158,$A8,'All Entries'!$E$2:$E$158,$B8,'All Entries'!$D$2:$D$158,$C8)</f>
         <v/>
       </c>
       <c r="J8" s="11">
@@ -784,27 +785,27 @@
         </is>
       </c>
       <c r="D9" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,D$4,'All Entries'!$C$2:$C$156,$A9,'All Entries'!$E$2:$E$156,$B9,'All Entries'!$D$2:$D$156,$C9)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,D$4,'All Entries'!$C$2:$C$158,$A9,'All Entries'!$E$2:$E$158,$B9,'All Entries'!$D$2:$D$158,$C9)</f>
         <v/>
       </c>
       <c r="E9" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,E$4,'All Entries'!$C$2:$C$156,$A9,'All Entries'!$E$2:$E$156,$B9,'All Entries'!$D$2:$D$156,$C9)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,E$4,'All Entries'!$C$2:$C$158,$A9,'All Entries'!$E$2:$E$158,$B9,'All Entries'!$D$2:$D$158,$C9)</f>
         <v/>
       </c>
       <c r="F9" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,F$4,'All Entries'!$C$2:$C$156,$A9,'All Entries'!$E$2:$E$156,$B9,'All Entries'!$D$2:$D$156,$C9)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,F$4,'All Entries'!$C$2:$C$158,$A9,'All Entries'!$E$2:$E$158,$B9,'All Entries'!$D$2:$D$158,$C9)</f>
         <v/>
       </c>
       <c r="G9" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,G$4,'All Entries'!$C$2:$C$156,$A9,'All Entries'!$E$2:$E$156,$B9,'All Entries'!$D$2:$D$156,$C9)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,G$4,'All Entries'!$C$2:$C$158,$A9,'All Entries'!$E$2:$E$158,$B9,'All Entries'!$D$2:$D$158,$C9)</f>
         <v/>
       </c>
       <c r="H9" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,H$4,'All Entries'!$C$2:$C$156,$A9,'All Entries'!$E$2:$E$156,$B9,'All Entries'!$D$2:$D$156,$C9)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,H$4,'All Entries'!$C$2:$C$158,$A9,'All Entries'!$E$2:$E$158,$B9,'All Entries'!$D$2:$D$158,$C9)</f>
         <v/>
       </c>
       <c r="I9" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,I$4,'All Entries'!$C$2:$C$156,$A9,'All Entries'!$E$2:$E$156,$B9,'All Entries'!$D$2:$D$156,$C9)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,I$4,'All Entries'!$C$2:$C$158,$A9,'All Entries'!$E$2:$E$158,$B9,'All Entries'!$D$2:$D$158,$C9)</f>
         <v/>
       </c>
       <c r="J9" s="11">
@@ -829,27 +830,27 @@
         </is>
       </c>
       <c r="D10" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,D$4,'All Entries'!$C$2:$C$156,$A10,'All Entries'!$E$2:$E$156,$B10,'All Entries'!$D$2:$D$156,$C10)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,D$4,'All Entries'!$C$2:$C$158,$A10,'All Entries'!$E$2:$E$158,$B10,'All Entries'!$D$2:$D$158,$C10)</f>
         <v/>
       </c>
       <c r="E10" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,E$4,'All Entries'!$C$2:$C$156,$A10,'All Entries'!$E$2:$E$156,$B10,'All Entries'!$D$2:$D$156,$C10)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,E$4,'All Entries'!$C$2:$C$158,$A10,'All Entries'!$E$2:$E$158,$B10,'All Entries'!$D$2:$D$158,$C10)</f>
         <v/>
       </c>
       <c r="F10" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,F$4,'All Entries'!$C$2:$C$156,$A10,'All Entries'!$E$2:$E$156,$B10,'All Entries'!$D$2:$D$156,$C10)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,F$4,'All Entries'!$C$2:$C$158,$A10,'All Entries'!$E$2:$E$158,$B10,'All Entries'!$D$2:$D$158,$C10)</f>
         <v/>
       </c>
       <c r="G10" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,G$4,'All Entries'!$C$2:$C$156,$A10,'All Entries'!$E$2:$E$156,$B10,'All Entries'!$D$2:$D$156,$C10)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,G$4,'All Entries'!$C$2:$C$158,$A10,'All Entries'!$E$2:$E$158,$B10,'All Entries'!$D$2:$D$158,$C10)</f>
         <v/>
       </c>
       <c r="H10" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,H$4,'All Entries'!$C$2:$C$156,$A10,'All Entries'!$E$2:$E$156,$B10,'All Entries'!$D$2:$D$156,$C10)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,H$4,'All Entries'!$C$2:$C$158,$A10,'All Entries'!$E$2:$E$158,$B10,'All Entries'!$D$2:$D$158,$C10)</f>
         <v/>
       </c>
       <c r="I10" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,I$4,'All Entries'!$C$2:$C$156,$A10,'All Entries'!$E$2:$E$156,$B10,'All Entries'!$D$2:$D$156,$C10)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,I$4,'All Entries'!$C$2:$C$158,$A10,'All Entries'!$E$2:$E$158,$B10,'All Entries'!$D$2:$D$158,$C10)</f>
         <v/>
       </c>
       <c r="J10" s="11">
@@ -874,27 +875,27 @@
         </is>
       </c>
       <c r="D11" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,D$4,'All Entries'!$C$2:$C$156,$A11,'All Entries'!$E$2:$E$156,$B11,'All Entries'!$D$2:$D$156,$C11)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,D$4,'All Entries'!$C$2:$C$158,$A11,'All Entries'!$E$2:$E$158,$B11,'All Entries'!$D$2:$D$158,$C11)</f>
         <v/>
       </c>
       <c r="E11" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,E$4,'All Entries'!$C$2:$C$156,$A11,'All Entries'!$E$2:$E$156,$B11,'All Entries'!$D$2:$D$156,$C11)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,E$4,'All Entries'!$C$2:$C$158,$A11,'All Entries'!$E$2:$E$158,$B11,'All Entries'!$D$2:$D$158,$C11)</f>
         <v/>
       </c>
       <c r="F11" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,F$4,'All Entries'!$C$2:$C$156,$A11,'All Entries'!$E$2:$E$156,$B11,'All Entries'!$D$2:$D$156,$C11)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,F$4,'All Entries'!$C$2:$C$158,$A11,'All Entries'!$E$2:$E$158,$B11,'All Entries'!$D$2:$D$158,$C11)</f>
         <v/>
       </c>
       <c r="G11" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,G$4,'All Entries'!$C$2:$C$156,$A11,'All Entries'!$E$2:$E$156,$B11,'All Entries'!$D$2:$D$156,$C11)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,G$4,'All Entries'!$C$2:$C$158,$A11,'All Entries'!$E$2:$E$158,$B11,'All Entries'!$D$2:$D$158,$C11)</f>
         <v/>
       </c>
       <c r="H11" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,H$4,'All Entries'!$C$2:$C$156,$A11,'All Entries'!$E$2:$E$156,$B11,'All Entries'!$D$2:$D$156,$C11)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,H$4,'All Entries'!$C$2:$C$158,$A11,'All Entries'!$E$2:$E$158,$B11,'All Entries'!$D$2:$D$158,$C11)</f>
         <v/>
       </c>
       <c r="I11" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,I$4,'All Entries'!$C$2:$C$156,$A11,'All Entries'!$E$2:$E$156,$B11,'All Entries'!$D$2:$D$156,$C11)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,I$4,'All Entries'!$C$2:$C$158,$A11,'All Entries'!$E$2:$E$158,$B11,'All Entries'!$D$2:$D$158,$C11)</f>
         <v/>
       </c>
       <c r="J11" s="11">
@@ -919,27 +920,27 @@
         </is>
       </c>
       <c r="D12" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,D$4,'All Entries'!$C$2:$C$156,$A12,'All Entries'!$E$2:$E$156,$B12,'All Entries'!$D$2:$D$156,$C12)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,D$4,'All Entries'!$C$2:$C$158,$A12,'All Entries'!$E$2:$E$158,$B12,'All Entries'!$D$2:$D$158,$C12)</f>
         <v/>
       </c>
       <c r="E12" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,E$4,'All Entries'!$C$2:$C$156,$A12,'All Entries'!$E$2:$E$156,$B12,'All Entries'!$D$2:$D$156,$C12)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,E$4,'All Entries'!$C$2:$C$158,$A12,'All Entries'!$E$2:$E$158,$B12,'All Entries'!$D$2:$D$158,$C12)</f>
         <v/>
       </c>
       <c r="F12" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,F$4,'All Entries'!$C$2:$C$156,$A12,'All Entries'!$E$2:$E$156,$B12,'All Entries'!$D$2:$D$156,$C12)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,F$4,'All Entries'!$C$2:$C$158,$A12,'All Entries'!$E$2:$E$158,$B12,'All Entries'!$D$2:$D$158,$C12)</f>
         <v/>
       </c>
       <c r="G12" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,G$4,'All Entries'!$C$2:$C$156,$A12,'All Entries'!$E$2:$E$156,$B12,'All Entries'!$D$2:$D$156,$C12)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,G$4,'All Entries'!$C$2:$C$158,$A12,'All Entries'!$E$2:$E$158,$B12,'All Entries'!$D$2:$D$158,$C12)</f>
         <v/>
       </c>
       <c r="H12" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,H$4,'All Entries'!$C$2:$C$156,$A12,'All Entries'!$E$2:$E$156,$B12,'All Entries'!$D$2:$D$156,$C12)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,H$4,'All Entries'!$C$2:$C$158,$A12,'All Entries'!$E$2:$E$158,$B12,'All Entries'!$D$2:$D$158,$C12)</f>
         <v/>
       </c>
       <c r="I12" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,I$4,'All Entries'!$C$2:$C$156,$A12,'All Entries'!$E$2:$E$156,$B12,'All Entries'!$D$2:$D$156,$C12)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,I$4,'All Entries'!$C$2:$C$158,$A12,'All Entries'!$E$2:$E$158,$B12,'All Entries'!$D$2:$D$158,$C12)</f>
         <v/>
       </c>
       <c r="J12" s="11">
@@ -964,27 +965,27 @@
         </is>
       </c>
       <c r="D13" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,D$4,'All Entries'!$C$2:$C$156,$A13,'All Entries'!$E$2:$E$156,$B13,'All Entries'!$D$2:$D$156,$C13)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,D$4,'All Entries'!$C$2:$C$158,$A13,'All Entries'!$E$2:$E$158,$B13,'All Entries'!$D$2:$D$158,$C13)</f>
         <v/>
       </c>
       <c r="E13" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,E$4,'All Entries'!$C$2:$C$156,$A13,'All Entries'!$E$2:$E$156,$B13,'All Entries'!$D$2:$D$156,$C13)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,E$4,'All Entries'!$C$2:$C$158,$A13,'All Entries'!$E$2:$E$158,$B13,'All Entries'!$D$2:$D$158,$C13)</f>
         <v/>
       </c>
       <c r="F13" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,F$4,'All Entries'!$C$2:$C$156,$A13,'All Entries'!$E$2:$E$156,$B13,'All Entries'!$D$2:$D$156,$C13)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,F$4,'All Entries'!$C$2:$C$158,$A13,'All Entries'!$E$2:$E$158,$B13,'All Entries'!$D$2:$D$158,$C13)</f>
         <v/>
       </c>
       <c r="G13" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,G$4,'All Entries'!$C$2:$C$156,$A13,'All Entries'!$E$2:$E$156,$B13,'All Entries'!$D$2:$D$156,$C13)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,G$4,'All Entries'!$C$2:$C$158,$A13,'All Entries'!$E$2:$E$158,$B13,'All Entries'!$D$2:$D$158,$C13)</f>
         <v/>
       </c>
       <c r="H13" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,H$4,'All Entries'!$C$2:$C$156,$A13,'All Entries'!$E$2:$E$156,$B13,'All Entries'!$D$2:$D$156,$C13)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,H$4,'All Entries'!$C$2:$C$158,$A13,'All Entries'!$E$2:$E$158,$B13,'All Entries'!$D$2:$D$158,$C13)</f>
         <v/>
       </c>
       <c r="I13" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,I$4,'All Entries'!$C$2:$C$156,$A13,'All Entries'!$E$2:$E$156,$B13,'All Entries'!$D$2:$D$156,$C13)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,I$4,'All Entries'!$C$2:$C$158,$A13,'All Entries'!$E$2:$E$158,$B13,'All Entries'!$D$2:$D$158,$C13)</f>
         <v/>
       </c>
       <c r="J13" s="11">
@@ -1009,27 +1010,27 @@
         </is>
       </c>
       <c r="D14" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,D$4,'All Entries'!$C$2:$C$156,$A14,'All Entries'!$E$2:$E$156,$B14,'All Entries'!$D$2:$D$156,$C14)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,D$4,'All Entries'!$C$2:$C$158,$A14,'All Entries'!$E$2:$E$158,$B14,'All Entries'!$D$2:$D$158,$C14)</f>
         <v/>
       </c>
       <c r="E14" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,E$4,'All Entries'!$C$2:$C$156,$A14,'All Entries'!$E$2:$E$156,$B14,'All Entries'!$D$2:$D$156,$C14)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,E$4,'All Entries'!$C$2:$C$158,$A14,'All Entries'!$E$2:$E$158,$B14,'All Entries'!$D$2:$D$158,$C14)</f>
         <v/>
       </c>
       <c r="F14" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,F$4,'All Entries'!$C$2:$C$156,$A14,'All Entries'!$E$2:$E$156,$B14,'All Entries'!$D$2:$D$156,$C14)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,F$4,'All Entries'!$C$2:$C$158,$A14,'All Entries'!$E$2:$E$158,$B14,'All Entries'!$D$2:$D$158,$C14)</f>
         <v/>
       </c>
       <c r="G14" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,G$4,'All Entries'!$C$2:$C$156,$A14,'All Entries'!$E$2:$E$156,$B14,'All Entries'!$D$2:$D$156,$C14)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,G$4,'All Entries'!$C$2:$C$158,$A14,'All Entries'!$E$2:$E$158,$B14,'All Entries'!$D$2:$D$158,$C14)</f>
         <v/>
       </c>
       <c r="H14" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,H$4,'All Entries'!$C$2:$C$156,$A14,'All Entries'!$E$2:$E$156,$B14,'All Entries'!$D$2:$D$156,$C14)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,H$4,'All Entries'!$C$2:$C$158,$A14,'All Entries'!$E$2:$E$158,$B14,'All Entries'!$D$2:$D$158,$C14)</f>
         <v/>
       </c>
       <c r="I14" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,I$4,'All Entries'!$C$2:$C$156,$A14,'All Entries'!$E$2:$E$156,$B14,'All Entries'!$D$2:$D$156,$C14)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,I$4,'All Entries'!$C$2:$C$158,$A14,'All Entries'!$E$2:$E$158,$B14,'All Entries'!$D$2:$D$158,$C14)</f>
         <v/>
       </c>
       <c r="J14" s="11">
@@ -1054,27 +1055,27 @@
         </is>
       </c>
       <c r="D15" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,D$4,'All Entries'!$C$2:$C$156,$A15,'All Entries'!$E$2:$E$156,$B15,'All Entries'!$D$2:$D$156,$C15)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,D$4,'All Entries'!$C$2:$C$158,$A15,'All Entries'!$E$2:$E$158,$B15,'All Entries'!$D$2:$D$158,$C15)</f>
         <v/>
       </c>
       <c r="E15" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,E$4,'All Entries'!$C$2:$C$156,$A15,'All Entries'!$E$2:$E$156,$B15,'All Entries'!$D$2:$D$156,$C15)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,E$4,'All Entries'!$C$2:$C$158,$A15,'All Entries'!$E$2:$E$158,$B15,'All Entries'!$D$2:$D$158,$C15)</f>
         <v/>
       </c>
       <c r="F15" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,F$4,'All Entries'!$C$2:$C$156,$A15,'All Entries'!$E$2:$E$156,$B15,'All Entries'!$D$2:$D$156,$C15)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,F$4,'All Entries'!$C$2:$C$158,$A15,'All Entries'!$E$2:$E$158,$B15,'All Entries'!$D$2:$D$158,$C15)</f>
         <v/>
       </c>
       <c r="G15" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,G$4,'All Entries'!$C$2:$C$156,$A15,'All Entries'!$E$2:$E$156,$B15,'All Entries'!$D$2:$D$156,$C15)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,G$4,'All Entries'!$C$2:$C$158,$A15,'All Entries'!$E$2:$E$158,$B15,'All Entries'!$D$2:$D$158,$C15)</f>
         <v/>
       </c>
       <c r="H15" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,H$4,'All Entries'!$C$2:$C$156,$A15,'All Entries'!$E$2:$E$156,$B15,'All Entries'!$D$2:$D$156,$C15)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,H$4,'All Entries'!$C$2:$C$158,$A15,'All Entries'!$E$2:$E$158,$B15,'All Entries'!$D$2:$D$158,$C15)</f>
         <v/>
       </c>
       <c r="I15" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,I$4,'All Entries'!$C$2:$C$156,$A15,'All Entries'!$E$2:$E$156,$B15,'All Entries'!$D$2:$D$156,$C15)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,I$4,'All Entries'!$C$2:$C$158,$A15,'All Entries'!$E$2:$E$158,$B15,'All Entries'!$D$2:$D$158,$C15)</f>
         <v/>
       </c>
       <c r="J15" s="11">
@@ -1099,27 +1100,27 @@
         </is>
       </c>
       <c r="D16" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,D$4,'All Entries'!$C$2:$C$156,$A16,'All Entries'!$E$2:$E$156,$B16,'All Entries'!$D$2:$D$156,$C16)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,D$4,'All Entries'!$C$2:$C$158,$A16,'All Entries'!$E$2:$E$158,$B16,'All Entries'!$D$2:$D$158,$C16)</f>
         <v/>
       </c>
       <c r="E16" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,E$4,'All Entries'!$C$2:$C$156,$A16,'All Entries'!$E$2:$E$156,$B16,'All Entries'!$D$2:$D$156,$C16)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,E$4,'All Entries'!$C$2:$C$158,$A16,'All Entries'!$E$2:$E$158,$B16,'All Entries'!$D$2:$D$158,$C16)</f>
         <v/>
       </c>
       <c r="F16" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,F$4,'All Entries'!$C$2:$C$156,$A16,'All Entries'!$E$2:$E$156,$B16,'All Entries'!$D$2:$D$156,$C16)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,F$4,'All Entries'!$C$2:$C$158,$A16,'All Entries'!$E$2:$E$158,$B16,'All Entries'!$D$2:$D$158,$C16)</f>
         <v/>
       </c>
       <c r="G16" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,G$4,'All Entries'!$C$2:$C$156,$A16,'All Entries'!$E$2:$E$156,$B16,'All Entries'!$D$2:$D$156,$C16)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,G$4,'All Entries'!$C$2:$C$158,$A16,'All Entries'!$E$2:$E$158,$B16,'All Entries'!$D$2:$D$158,$C16)</f>
         <v/>
       </c>
       <c r="H16" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,H$4,'All Entries'!$C$2:$C$156,$A16,'All Entries'!$E$2:$E$156,$B16,'All Entries'!$D$2:$D$156,$C16)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,H$4,'All Entries'!$C$2:$C$158,$A16,'All Entries'!$E$2:$E$158,$B16,'All Entries'!$D$2:$D$158,$C16)</f>
         <v/>
       </c>
       <c r="I16" s="9">
-        <f>COUNTIFS('All Entries'!$B$2:$B$156,I$4,'All Entries'!$C$2:$C$156,$A16,'All Entries'!$E$2:$E$156,$B16,'All Entries'!$D$2:$D$156,$C16)</f>
+        <f>COUNTIFS('All Entries'!$B$2:$B$158,I$4,'All Entries'!$C$2:$C$158,$A16,'All Entries'!$E$2:$E$158,$B16,'All Entries'!$D$2:$D$158,$C16)</f>
         <v/>
       </c>
       <c r="J16" s="11">
@@ -1173,22 +1174,22 @@
       <c r="B18" s="12" t="n"/>
       <c r="C18" s="12" t="n"/>
       <c r="D18" s="14" t="n">
+        <v>17</v>
+      </c>
+      <c r="E18" s="14" t="n">
         <v>18</v>
       </c>
-      <c r="E18" s="14" t="n">
-        <v>19</v>
-      </c>
       <c r="F18" s="14" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H18" s="14" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I18" s="14" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J18" s="14" t="n"/>
     </row>
@@ -2198,7 +2199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H156"/>
+  <dimension ref="A1:H158"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="5" customWidth="1" style="15" min="1" max="1"/>
@@ -2349,7 +2350,7 @@
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
-          <t>Gokul</t>
+          <t>Amal Jose</t>
         </is>
       </c>
       <c r="G4" s="10" t="n"/>
@@ -2384,7 +2385,7 @@
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>Amal</t>
+          <t>Gokul K R</t>
         </is>
       </c>
       <c r="G5" s="10" t="n"/>
@@ -2419,7 +2420,7 @@
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>Kevin</t>
+          <t>Kevin Raj</t>
         </is>
       </c>
       <c r="G6" s="10" t="n"/>
@@ -2454,7 +2455,7 @@
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>Adwaith</t>
+          <t>Adwaith Narayanan</t>
         </is>
       </c>
       <c r="G7" s="10" t="n"/>
@@ -2489,7 +2490,7 @@
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>Sahil M I</t>
+          <t>Anandhan Sreekumar</t>
         </is>
       </c>
       <c r="G8" s="10" t="n"/>
@@ -2524,7 +2525,7 @@
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>Rajeesh C V</t>
+          <t>Soorya Thejas</t>
         </is>
       </c>
       <c r="G9" s="10" t="n"/>
@@ -2559,7 +2560,7 @@
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>Adhith Vinoj</t>
+          <t>Nidheesh P V</t>
         </is>
       </c>
       <c r="G10" s="10" t="n"/>
@@ -2594,7 +2595,7 @@
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>Nidheesh P V</t>
+          <t>Adhith Vinoj</t>
         </is>
       </c>
       <c r="G11" s="10" t="n"/>
@@ -2629,7 +2630,7 @@
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>Joel</t>
+          <t>Joel Paul</t>
         </is>
       </c>
       <c r="G12" s="10" t="n"/>
@@ -2664,7 +2665,7 @@
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>Jayesh</t>
+          <t>Musthaq</t>
         </is>
       </c>
       <c r="G13" s="10" t="n"/>
@@ -2734,7 +2735,7 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Nivya</t>
+          <t>Nivya Mathew</t>
         </is>
       </c>
       <c r="G15" s="10" t="n"/>
@@ -2769,7 +2770,7 @@
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>Tressy</t>
+          <t>Anima V Shaji</t>
         </is>
       </c>
       <c r="G16" s="10" t="n"/>
@@ -2804,7 +2805,7 @@
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>Anima</t>
+          <t>Tressy</t>
         </is>
       </c>
       <c r="G17" s="10" t="n"/>
@@ -2839,7 +2840,7 @@
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>Anjaly</t>
+          <t>Anjaly C Prakash</t>
         </is>
       </c>
       <c r="G18" s="10" t="n"/>
@@ -2874,7 +2875,7 @@
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Fadwah</t>
+          <t>Neha Abdul Majeed</t>
         </is>
       </c>
       <c r="G19" s="10" t="n"/>
@@ -3084,7 +3085,7 @@
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>Akshaya</t>
+          <t>Ashna</t>
         </is>
       </c>
       <c r="G25" s="10" t="n"/>
@@ -3163,7 +3164,7 @@
       </c>
       <c r="G27" s="10" t="inlineStr">
         <is>
-          <t>Jithu</t>
+          <t>Shamil</t>
         </is>
       </c>
       <c r="H27" s="10">
@@ -3197,12 +3198,12 @@
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>Gokul</t>
+          <t>Amal Jose</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>Amal</t>
+          <t>Gokul K R</t>
         </is>
       </c>
       <c r="H28" s="10">
@@ -3241,7 +3242,7 @@
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
-          <t>Sravan</t>
+          <t>Boban Paul</t>
         </is>
       </c>
       <c r="H29" s="10">
@@ -3275,12 +3276,12 @@
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t>Ashmil</t>
+          <t>Kevin Raj</t>
         </is>
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>Jerishab</t>
+          <t>Adwaith Narayanan</t>
         </is>
       </c>
       <c r="H30" s="10">
@@ -3314,12 +3315,12 @@
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
-          <t>Rithik</t>
+          <t>Rithik P Vijay</t>
         </is>
       </c>
       <c r="G31" s="10" t="inlineStr">
         <is>
-          <t>Jerin</t>
+          <t>Jerin Wilson</t>
         </is>
       </c>
       <c r="H31" s="10">
@@ -3353,12 +3354,12 @@
       </c>
       <c r="F32" s="10" t="inlineStr">
         <is>
-          <t>Sahil M I</t>
+          <t>Rajeesh C V</t>
         </is>
       </c>
       <c r="G32" s="10" t="inlineStr">
         <is>
-          <t>Rajeesh C V</t>
+          <t>Akhil P Jose</t>
         </is>
       </c>
       <c r="H32" s="10">
@@ -3392,7 +3393,7 @@
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
-          <t>Don</t>
+          <t>Sahil M I</t>
         </is>
       </c>
       <c r="G33" s="10" t="inlineStr">
@@ -3450,7 +3451,7 @@
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Team 6 – Aaram Thamburan</t>
+          <t>Team 5 – Dhurandhar</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
@@ -3470,12 +3471,12 @@
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
-          <t>Joel</t>
+          <t>Abhijith K V</t>
         </is>
       </c>
       <c r="G35" s="10" t="inlineStr">
         <is>
-          <t>Jayesh</t>
+          <t>Akshay A</t>
         </is>
       </c>
       <c r="H35" s="10">
@@ -3509,7 +3510,7 @@
       </c>
       <c r="F36" s="10" t="inlineStr">
         <is>
-          <t>Sharan</t>
+          <t>Joel Paul</t>
         </is>
       </c>
       <c r="G36" s="10" t="inlineStr">
@@ -3528,7 +3529,7 @@
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>Team 1 – Rajarajeshwari United</t>
+          <t>Team 6 – Aaram Thamburan</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
@@ -3538,7 +3539,7 @@
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>Women</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
@@ -3548,12 +3549,12 @@
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
-          <t>Neethu</t>
+          <t>Jayesh</t>
         </is>
       </c>
       <c r="G37" s="10" t="inlineStr">
         <is>
-          <t>Nivya Mathew</t>
+          <t>Ansam</t>
         </is>
       </c>
       <c r="H37" s="10">
@@ -3587,12 +3588,12 @@
       </c>
       <c r="F38" s="10" t="inlineStr">
         <is>
-          <t>Nivya Peter</t>
+          <t>Neethu</t>
         </is>
       </c>
       <c r="G38" s="10" t="inlineStr">
         <is>
-          <t>Bilsy</t>
+          <t>Nivya Mathew</t>
         </is>
       </c>
       <c r="H38" s="10">
@@ -3606,7 +3607,7 @@
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>Team 2 – Jeem Boom Baa</t>
+          <t>Team 1 – Rajarajeshwari United</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
@@ -3626,12 +3627,12 @@
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
-          <t>Tressy</t>
+          <t>Shinu</t>
         </is>
       </c>
       <c r="G39" s="10" t="inlineStr">
         <is>
-          <t>Anima</t>
+          <t>Bilsy</t>
         </is>
       </c>
       <c r="H39" s="10">
@@ -3665,12 +3666,12 @@
       </c>
       <c r="F40" s="10" t="inlineStr">
         <is>
-          <t>Surya</t>
+          <t>Josna Mathew</t>
         </is>
       </c>
       <c r="G40" s="10" t="inlineStr">
         <is>
-          <t>Josna</t>
+          <t>Athira Jayaprasad</t>
         </is>
       </c>
       <c r="H40" s="10">
@@ -3684,7 +3685,7 @@
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 2 – Jeem Boom Baa</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
@@ -3704,12 +3705,12 @@
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
-          <t>Anjaly</t>
+          <t>Anima V Shaji</t>
         </is>
       </c>
       <c r="G41" s="10" t="inlineStr">
         <is>
-          <t>Fadwah</t>
+          <t>Tressy</t>
         </is>
       </c>
       <c r="H41" s="10">
@@ -3743,12 +3744,12 @@
       </c>
       <c r="F42" s="10" t="inlineStr">
         <is>
-          <t>Neha</t>
+          <t>Anjaly C Prakash</t>
         </is>
       </c>
       <c r="G42" s="10" t="inlineStr">
         <is>
-          <t>Nandana</t>
+          <t>Anan Nasreen</t>
         </is>
       </c>
       <c r="H42" s="10">
@@ -3762,7 +3763,7 @@
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>Team 4 – Thoofan</t>
+          <t>Team 3 – Dr. D</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
@@ -3782,12 +3783,12 @@
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
-          <t>Manjusha</t>
+          <t>Neha Abdul Majeed</t>
         </is>
       </c>
       <c r="G43" s="10" t="inlineStr">
         <is>
-          <t>AnnMary</t>
+          <t>Nandhana Rayaroth</t>
         </is>
       </c>
       <c r="H43" s="10">
@@ -3821,12 +3822,12 @@
       </c>
       <c r="F44" s="10" t="inlineStr">
         <is>
-          <t>Aparna</t>
+          <t>Manjusha</t>
         </is>
       </c>
       <c r="G44" s="10" t="inlineStr">
         <is>
-          <t>Gayathri</t>
+          <t>AnnMary</t>
         </is>
       </c>
       <c r="H44" s="10">
@@ -3840,7 +3841,7 @@
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>Team 5 – Dhurandhar</t>
+          <t>Team 4 – Thoofan</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
@@ -3860,12 +3861,12 @@
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
-          <t>Sradha Santhosh</t>
+          <t>Aparna</t>
         </is>
       </c>
       <c r="G45" s="10" t="inlineStr">
         <is>
-          <t>Vidhya M Robert</t>
+          <t>Gayathri</t>
         </is>
       </c>
       <c r="H45" s="10">
@@ -3879,7 +3880,7 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>Team 6 – Aaram Thamburan</t>
+          <t>Team 5 – Dhurandhar</t>
         </is>
       </c>
       <c r="C46" s="10" t="inlineStr">
@@ -3899,12 +3900,12 @@
       </c>
       <c r="F46" s="10" t="inlineStr">
         <is>
-          <t>Merrin</t>
+          <t>Riya Fathima</t>
         </is>
       </c>
       <c r="G46" s="10" t="inlineStr">
         <is>
-          <t>Akshaya</t>
+          <t>Ameesha T</t>
         </is>
       </c>
       <c r="H46" s="10">
@@ -3918,7 +3919,7 @@
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>Team 6 – Aaram Thamburan</t>
+          <t>Team 5 – Dhurandhar</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
@@ -3938,12 +3939,12 @@
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
-          <t>Ashna</t>
+          <t>Sradha Santhosh</t>
         </is>
       </c>
       <c r="G47" s="10" t="inlineStr">
         <is>
-          <t>Akhila / Athira</t>
+          <t>Vidhya M Robert</t>
         </is>
       </c>
       <c r="H47" s="10">
@@ -3957,30 +3958,34 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>Team 1 – Rajarajeshwari United</t>
+          <t>Team 6 – Aaram Thamburan</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>Table Tennis</t>
+          <t>Badminton</t>
         </is>
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t>Men</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="E48" s="10" t="inlineStr">
         <is>
-          <t>Singles</t>
+          <t>Doubles</t>
         </is>
       </c>
       <c r="F48" s="10" t="inlineStr">
         <is>
-          <t>Rishikesh</t>
-        </is>
-      </c>
-      <c r="G48" s="10" t="n"/>
+          <t>Merrin</t>
+        </is>
+      </c>
+      <c r="G48" s="10" t="inlineStr">
+        <is>
+          <t>Ashna</t>
+        </is>
+      </c>
       <c r="H48" s="10">
         <f>IF(G48="",F48,F48&amp;" &amp; "&amp;G48)</f>
         <v/>
@@ -3992,30 +3997,34 @@
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>Team 1 – Rajarajeshwari United</t>
+          <t>Team 6 – Aaram Thamburan</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>Table Tennis</t>
+          <t>Badminton</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>Men</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="E49" s="10" t="inlineStr">
         <is>
-          <t>Singles</t>
+          <t>Doubles</t>
         </is>
       </c>
       <c r="F49" s="10" t="inlineStr">
         <is>
-          <t>Amit</t>
-        </is>
-      </c>
-      <c r="G49" s="10" t="n"/>
+          <t>Akshaya</t>
+        </is>
+      </c>
+      <c r="G49" s="10" t="inlineStr">
+        <is>
+          <t>Athira</t>
+        </is>
+      </c>
       <c r="H49" s="10">
         <f>IF(G49="",F49,F49&amp;" &amp; "&amp;G49)</f>
         <v/>
@@ -4047,7 +4056,7 @@
       </c>
       <c r="F50" s="10" t="inlineStr">
         <is>
-          <t>Bilal</t>
+          <t>Rishikesh</t>
         </is>
       </c>
       <c r="G50" s="10" t="n"/>
@@ -4082,7 +4091,7 @@
       </c>
       <c r="F51" s="10" t="inlineStr">
         <is>
-          <t>Deekshith</t>
+          <t>Amit</t>
         </is>
       </c>
       <c r="G51" s="10" t="n"/>
@@ -4117,7 +4126,7 @@
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
-          <t>Joyel</t>
+          <t>Bilal</t>
         </is>
       </c>
       <c r="G52" s="10" t="n"/>
@@ -4152,7 +4161,7 @@
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
-          <t>Vidhu</t>
+          <t>Deekshith</t>
         </is>
       </c>
       <c r="G53" s="10" t="n"/>
@@ -4167,7 +4176,7 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>Team 2 – Jeem Boom Baa</t>
+          <t>Team 1 – Rajarajeshwari United</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
@@ -4187,7 +4196,7 @@
       </c>
       <c r="F54" s="10" t="inlineStr">
         <is>
-          <t>Ray</t>
+          <t>Joyel</t>
         </is>
       </c>
       <c r="G54" s="10" t="n"/>
@@ -4202,7 +4211,7 @@
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>Team 2 – Jeem Boom Baa</t>
+          <t>Team 1 – Rajarajeshwari United</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
@@ -4222,7 +4231,7 @@
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Vidhu</t>
         </is>
       </c>
       <c r="G55" s="10" t="n"/>
@@ -4237,7 +4246,7 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 2 – Jeem Boom Baa</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
@@ -4257,7 +4266,7 @@
       </c>
       <c r="F56" s="10" t="inlineStr">
         <is>
-          <t>Rithik</t>
+          <t>Ray</t>
         </is>
       </c>
       <c r="G56" s="10" t="n"/>
@@ -4272,7 +4281,7 @@
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 2 – Jeem Boom Baa</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
@@ -4292,7 +4301,7 @@
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
-          <t>Alwin</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="G57" s="10" t="n"/>
@@ -4327,7 +4336,7 @@
       </c>
       <c r="F58" s="10" t="inlineStr">
         <is>
-          <t>Adwaith</t>
+          <t>Rithik P Vijay</t>
         </is>
       </c>
       <c r="G58" s="10" t="n"/>
@@ -4362,7 +4371,7 @@
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
-          <t>Prajith</t>
+          <t>Alwin</t>
         </is>
       </c>
       <c r="G59" s="10" t="n"/>
@@ -4397,7 +4406,7 @@
       </c>
       <c r="F60" s="10" t="inlineStr">
         <is>
-          <t>Nived</t>
+          <t>Adwaith Narayanan</t>
         </is>
       </c>
       <c r="G60" s="10" t="n"/>
@@ -4412,7 +4421,7 @@
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>Team 4 – Thoofan</t>
+          <t>Team 3 – Dr. D</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
@@ -4432,7 +4441,7 @@
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
-          <t>Sahil M I</t>
+          <t>Prajith</t>
         </is>
       </c>
       <c r="G61" s="10" t="n"/>
@@ -4447,7 +4456,7 @@
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>Team 4 – Thoofan</t>
+          <t>Team 3 – Dr. D</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
@@ -4467,7 +4476,7 @@
       </c>
       <c r="F62" s="10" t="inlineStr">
         <is>
-          <t>Suryathejas</t>
+          <t>Nived</t>
         </is>
       </c>
       <c r="G62" s="10" t="n"/>
@@ -4502,7 +4511,7 @@
       </c>
       <c r="F63" s="10" t="inlineStr">
         <is>
-          <t>Rajeesh C V</t>
+          <t>Sahil M I</t>
         </is>
       </c>
       <c r="G63" s="10" t="n"/>
@@ -4537,7 +4546,7 @@
       </c>
       <c r="F64" s="10" t="inlineStr">
         <is>
-          <t>Subin</t>
+          <t>Soorya Thejas</t>
         </is>
       </c>
       <c r="G64" s="10" t="n"/>
@@ -4572,7 +4581,7 @@
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
-          <t>Arshal Abbas</t>
+          <t>Rajeesh C V</t>
         </is>
       </c>
       <c r="G65" s="10" t="n"/>
@@ -4587,7 +4596,7 @@
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>Team 5 – Dhurandhar</t>
+          <t>Team 4 – Thoofan</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
@@ -4607,7 +4616,7 @@
       </c>
       <c r="F66" s="10" t="inlineStr">
         <is>
-          <t>Nidheesh P V</t>
+          <t>Subin</t>
         </is>
       </c>
       <c r="G66" s="10" t="n"/>
@@ -4622,7 +4631,7 @@
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>Team 5 – Dhurandhar</t>
+          <t>Team 4 – Thoofan</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
@@ -4642,7 +4651,7 @@
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
-          <t>Abhishek P S</t>
+          <t>Arshal Abbas</t>
         </is>
       </c>
       <c r="G67" s="10" t="n"/>
@@ -4657,7 +4666,7 @@
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>Team 6 – Aaram Thamburan</t>
+          <t>Team 5 – Dhurandhar</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
@@ -4677,7 +4686,7 @@
       </c>
       <c r="F68" s="10" t="inlineStr">
         <is>
-          <t>Ansam</t>
+          <t>Nidheesh P V</t>
         </is>
       </c>
       <c r="G68" s="10" t="n"/>
@@ -4692,7 +4701,7 @@
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>Team 6 – Aaram Thamburan</t>
+          <t>Team 5 – Dhurandhar</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
@@ -4712,7 +4721,7 @@
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
-          <t>Musthaq</t>
+          <t>Abhishek P S</t>
         </is>
       </c>
       <c r="G69" s="10" t="n"/>
@@ -4727,7 +4736,7 @@
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>Team 1 – Rajarajeshwari United</t>
+          <t>Team 6 – Aaram Thamburan</t>
         </is>
       </c>
       <c r="C70" s="10" t="inlineStr">
@@ -4737,7 +4746,7 @@
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t>Women</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="E70" s="10" t="inlineStr">
@@ -4747,7 +4756,7 @@
       </c>
       <c r="F70" s="10" t="inlineStr">
         <is>
-          <t>Neethu</t>
+          <t>Ansam</t>
         </is>
       </c>
       <c r="G70" s="10" t="n"/>
@@ -4762,7 +4771,7 @@
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>Team 1 – Rajarajeshwari United</t>
+          <t>Team 6 – Aaram Thamburan</t>
         </is>
       </c>
       <c r="C71" s="10" t="inlineStr">
@@ -4772,7 +4781,7 @@
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t>Women</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="E71" s="10" t="inlineStr">
@@ -4782,7 +4791,7 @@
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
-          <t>Nivya Mathew</t>
+          <t>Musthaq</t>
         </is>
       </c>
       <c r="G71" s="10" t="n"/>
@@ -4797,7 +4806,7 @@
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 1 – Rajarajeshwari United</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
@@ -4817,7 +4826,7 @@
       </c>
       <c r="F72" s="10" t="inlineStr">
         <is>
-          <t>Anan</t>
+          <t>Neethu</t>
         </is>
       </c>
       <c r="G72" s="10" t="n"/>
@@ -4832,7 +4841,7 @@
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>Team 4 – Thoofan</t>
+          <t>Team 1 – Rajarajeshwari United</t>
         </is>
       </c>
       <c r="C73" s="10" t="inlineStr">
@@ -4852,7 +4861,7 @@
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
-          <t>Deepanjali</t>
+          <t>Nivya Mathew</t>
         </is>
       </c>
       <c r="G73" s="10" t="n"/>
@@ -4867,7 +4876,7 @@
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t>Team 4 – Thoofan</t>
+          <t>Team 3 – Dr. D</t>
         </is>
       </c>
       <c r="C74" s="10" t="inlineStr">
@@ -4887,7 +4896,7 @@
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t>Aparna</t>
+          <t>Anan Nasreen</t>
         </is>
       </c>
       <c r="G74" s="10" t="n"/>
@@ -4902,7 +4911,7 @@
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t>Team 5 – Dhurandhar</t>
+          <t>Team 4 – Thoofan</t>
         </is>
       </c>
       <c r="C75" s="10" t="inlineStr">
@@ -4922,7 +4931,7 @@
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
-          <t>Sradha Santhosh</t>
+          <t>Deepanjali</t>
         </is>
       </c>
       <c r="G75" s="10" t="n"/>
@@ -4937,7 +4946,7 @@
       </c>
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t>Team 6 – Aaram Thamburan</t>
+          <t>Team 4 – Thoofan</t>
         </is>
       </c>
       <c r="C76" s="10" t="inlineStr">
@@ -4957,7 +4966,7 @@
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
-          <t>Akhila</t>
+          <t>Aparna</t>
         </is>
       </c>
       <c r="G76" s="10" t="n"/>
@@ -4972,7 +4981,7 @@
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t>Team 6 – Aaram Thamburan</t>
+          <t>Team 5 – Dhurandhar</t>
         </is>
       </c>
       <c r="C77" s="10" t="inlineStr">
@@ -4992,7 +5001,7 @@
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
-          <t>Ashna</t>
+          <t>Sradha Santhosh</t>
         </is>
       </c>
       <c r="G77" s="10" t="n"/>
@@ -5007,7 +5016,7 @@
       </c>
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t>Team 1 – Rajarajeshwari United</t>
+          <t>Team 6 – Aaram Thamburan</t>
         </is>
       </c>
       <c r="C78" s="10" t="inlineStr">
@@ -5017,24 +5026,20 @@
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t>Men</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="E78" s="10" t="inlineStr">
         <is>
-          <t>Doubles</t>
+          <t>Singles</t>
         </is>
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
-          <t>Rishikesh</t>
-        </is>
-      </c>
-      <c r="G78" s="10" t="inlineStr">
-        <is>
-          <t>Amit</t>
-        </is>
-      </c>
+          <t>Akhila</t>
+        </is>
+      </c>
+      <c r="G78" s="10" t="n"/>
       <c r="H78" s="10">
         <f>IF(G78="",F78,F78&amp;" &amp; "&amp;G78)</f>
         <v/>
@@ -5046,7 +5051,7 @@
       </c>
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t>Team 1 – Rajarajeshwari United</t>
+          <t>Team 6 – Aaram Thamburan</t>
         </is>
       </c>
       <c r="C79" s="10" t="inlineStr">
@@ -5056,24 +5061,20 @@
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t>Men</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="E79" s="10" t="inlineStr">
         <is>
-          <t>Doubles</t>
+          <t>Singles</t>
         </is>
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
-          <t>Bilal</t>
-        </is>
-      </c>
-      <c r="G79" s="10" t="inlineStr">
-        <is>
-          <t>Deekshith</t>
-        </is>
-      </c>
+          <t>Ashna</t>
+        </is>
+      </c>
+      <c r="G79" s="10" t="n"/>
       <c r="H79" s="10">
         <f>IF(G79="",F79,F79&amp;" &amp; "&amp;G79)</f>
         <v/>
@@ -5105,12 +5106,12 @@
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
-          <t>Joyel</t>
+          <t>Rishikesh</t>
         </is>
       </c>
       <c r="G80" s="10" t="inlineStr">
         <is>
-          <t>Vidhu</t>
+          <t>Amit</t>
         </is>
       </c>
       <c r="H80" s="10">
@@ -5124,7 +5125,7 @@
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>Team 2 – Jeem Boom Baa</t>
+          <t>Team 1 – Rajarajeshwari United</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
@@ -5144,12 +5145,12 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Bilal</t>
         </is>
       </c>
       <c r="G81" s="10" t="inlineStr">
         <is>
-          <t>Ray</t>
+          <t>Deekshith</t>
         </is>
       </c>
       <c r="H81" s="10">
@@ -5163,7 +5164,7 @@
       </c>
       <c r="B82" s="10" t="inlineStr">
         <is>
-          <t>Team 2 – Jeem Boom Baa</t>
+          <t>Team 1 – Rajarajeshwari United</t>
         </is>
       </c>
       <c r="C82" s="10" t="inlineStr">
@@ -5183,12 +5184,12 @@
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
-          <t>Bonny</t>
+          <t>Joyel</t>
         </is>
       </c>
       <c r="G82" s="10" t="inlineStr">
         <is>
-          <t>Akshay</t>
+          <t>Vidhu</t>
         </is>
       </c>
       <c r="H82" s="10">
@@ -5202,7 +5203,7 @@
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 2 – Jeem Boom Baa</t>
         </is>
       </c>
       <c r="C83" s="10" t="inlineStr">
@@ -5222,12 +5223,12 @@
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
-          <t>Adwaith</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="G83" s="10" t="inlineStr">
         <is>
-          <t>Alwin</t>
+          <t>Ray</t>
         </is>
       </c>
       <c r="H83" s="10">
@@ -5241,7 +5242,7 @@
       </c>
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 2 – Jeem Boom Baa</t>
         </is>
       </c>
       <c r="C84" s="10" t="inlineStr">
@@ -5261,12 +5262,12 @@
       </c>
       <c r="F84" s="10" t="inlineStr">
         <is>
-          <t>Prajith</t>
+          <t>Bonny</t>
         </is>
       </c>
       <c r="G84" s="10" t="inlineStr">
         <is>
-          <t>Nived</t>
+          <t>Akshay</t>
         </is>
       </c>
       <c r="H84" s="10">
@@ -5300,12 +5301,12 @@
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
-          <t>Rithik</t>
+          <t>Adwaith Narayanan</t>
         </is>
       </c>
       <c r="G85" s="10" t="inlineStr">
         <is>
-          <t>Prathyush</t>
+          <t>Alwin</t>
         </is>
       </c>
       <c r="H85" s="10">
@@ -5319,7 +5320,7 @@
       </c>
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t>Team 4 – Thoofan</t>
+          <t>Team 3 – Dr. D</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
@@ -5339,12 +5340,12 @@
       </c>
       <c r="F86" s="10" t="inlineStr">
         <is>
-          <t>Rajeesh C V</t>
+          <t>Prajith</t>
         </is>
       </c>
       <c r="G86" s="10" t="inlineStr">
         <is>
-          <t>Suryathejas</t>
+          <t>Nived</t>
         </is>
       </c>
       <c r="H86" s="10">
@@ -5358,7 +5359,7 @@
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t>Team 4 – Thoofan</t>
+          <t>Team 3 – Dr. D</t>
         </is>
       </c>
       <c r="C87" s="10" t="inlineStr">
@@ -5378,12 +5379,12 @@
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
-          <t>Subin</t>
+          <t>Rithik P Vijay</t>
         </is>
       </c>
       <c r="G87" s="10" t="inlineStr">
         <is>
-          <t>Sahil M I</t>
+          <t>Prathyush</t>
         </is>
       </c>
       <c r="H87" s="10">
@@ -5397,7 +5398,7 @@
       </c>
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t>Team 5 – Dhurandhar</t>
+          <t>Team 4 – Thoofan</t>
         </is>
       </c>
       <c r="C88" s="10" t="inlineStr">
@@ -5417,12 +5418,12 @@
       </c>
       <c r="F88" s="10" t="inlineStr">
         <is>
-          <t>Nidheesh P V</t>
+          <t>Rajeesh C V</t>
         </is>
       </c>
       <c r="G88" s="10" t="inlineStr">
         <is>
-          <t>Abhishek P S</t>
+          <t>Soorya Thejas</t>
         </is>
       </c>
       <c r="H88" s="10">
@@ -5436,7 +5437,7 @@
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t>Team 6 – Aaram Thamburan</t>
+          <t>Team 4 – Thoofan</t>
         </is>
       </c>
       <c r="C89" s="10" t="inlineStr">
@@ -5456,12 +5457,12 @@
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
-          <t>Ansam</t>
+          <t>Subin</t>
         </is>
       </c>
       <c r="G89" s="10" t="inlineStr">
         <is>
-          <t>Musthaq</t>
+          <t>Sahil M I</t>
         </is>
       </c>
       <c r="H89" s="10">
@@ -5475,7 +5476,7 @@
       </c>
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t>Team 6 – Aaram Thamburan</t>
+          <t>Team 5 – Dhurandhar</t>
         </is>
       </c>
       <c r="C90" s="10" t="inlineStr">
@@ -5495,12 +5496,12 @@
       </c>
       <c r="F90" s="10" t="inlineStr">
         <is>
-          <t>Anandhakrishnan</t>
+          <t>Nidheesh P V</t>
         </is>
       </c>
       <c r="G90" s="10" t="inlineStr">
         <is>
-          <t>Christo</t>
+          <t>Abhishek P S</t>
         </is>
       </c>
       <c r="H90" s="10">
@@ -5514,7 +5515,7 @@
       </c>
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t>Team 1 – Rajarajeshwari United</t>
+          <t>Team 6 – Aaram Thamburan</t>
         </is>
       </c>
       <c r="C91" s="10" t="inlineStr">
@@ -5524,7 +5525,7 @@
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t>Women</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="E91" s="10" t="inlineStr">
@@ -5534,12 +5535,12 @@
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
-          <t>Neethu</t>
+          <t>Ansam</t>
         </is>
       </c>
       <c r="G91" s="10" t="inlineStr">
         <is>
-          <t>Nivya Mathew</t>
+          <t>Musthaq</t>
         </is>
       </c>
       <c r="H91" s="10">
@@ -5553,7 +5554,7 @@
       </c>
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t>Team 4 – Thoofan</t>
+          <t>Team 6 – Aaram Thamburan</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
@@ -5563,7 +5564,7 @@
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t>Women</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="E92" s="10" t="inlineStr">
@@ -5573,12 +5574,12 @@
       </c>
       <c r="F92" s="10" t="inlineStr">
         <is>
-          <t>Aparna</t>
+          <t>Anandhakrishnan</t>
         </is>
       </c>
       <c r="G92" s="10" t="inlineStr">
         <is>
-          <t>Deepanjali</t>
+          <t>Christo</t>
         </is>
       </c>
       <c r="H92" s="10">
@@ -5592,7 +5593,7 @@
       </c>
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t>Team 5 – Dhurandhar</t>
+          <t>Team 1 – Rajarajeshwari United</t>
         </is>
       </c>
       <c r="C93" s="10" t="inlineStr">
@@ -5612,12 +5613,12 @@
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
-          <t>Sradha Santhosh</t>
+          <t>Neethu</t>
         </is>
       </c>
       <c r="G93" s="10" t="inlineStr">
         <is>
-          <t>Aryamol</t>
+          <t>Nivya Mathew</t>
         </is>
       </c>
       <c r="H93" s="10">
@@ -5631,7 +5632,7 @@
       </c>
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t>Team 6 – Aaram Thamburan</t>
+          <t>Team 4 – Thoofan</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
@@ -5651,12 +5652,12 @@
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t>Akhila</t>
+          <t>Aparna</t>
         </is>
       </c>
       <c r="G94" s="10" t="inlineStr">
         <is>
-          <t>Ashna</t>
+          <t>Deepanjali</t>
         </is>
       </c>
       <c r="H94" s="10">
@@ -5670,17 +5671,17 @@
       </c>
       <c r="B95" s="10" t="inlineStr">
         <is>
-          <t>Team 1 – Rajarajeshwari United</t>
+          <t>Team 5 – Dhurandhar</t>
         </is>
       </c>
       <c r="C95" s="10" t="inlineStr">
         <is>
-          <t>Carrom</t>
+          <t>Table Tennis</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="E95" s="10" t="inlineStr">
@@ -5690,12 +5691,12 @@
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t>Joyel</t>
+          <t>Sradha Santhosh</t>
         </is>
       </c>
       <c r="G95" s="10" t="inlineStr">
         <is>
-          <t>Shinu</t>
+          <t>Aryamol</t>
         </is>
       </c>
       <c r="H95" s="10">
@@ -5709,17 +5710,17 @@
       </c>
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t>Team 1 – Rajarajeshwari United</t>
+          <t>Team 6 – Aaram Thamburan</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
         <is>
-          <t>Carrom</t>
+          <t>Table Tennis</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="E96" s="10" t="inlineStr">
@@ -5729,12 +5730,12 @@
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
-          <t>Deekshith</t>
+          <t>Akhila</t>
         </is>
       </c>
       <c r="G96" s="10" t="inlineStr">
         <is>
-          <t>Akshay</t>
+          <t>Ashna</t>
         </is>
       </c>
       <c r="H96" s="10">
@@ -5768,12 +5769,12 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t>Sharon</t>
+          <t>Joyel</t>
         </is>
       </c>
       <c r="G97" s="10" t="inlineStr">
         <is>
-          <t>Amit</t>
+          <t>Shinu</t>
         </is>
       </c>
       <c r="H97" s="10">
@@ -5807,12 +5808,12 @@
       </c>
       <c r="F98" s="10" t="inlineStr">
         <is>
-          <t>Neethu</t>
+          <t>Deekshith</t>
         </is>
       </c>
       <c r="G98" s="10" t="inlineStr">
         <is>
-          <t>Vidhu</t>
+          <t>Akshay</t>
         </is>
       </c>
       <c r="H98" s="10">
@@ -5846,12 +5847,12 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>Nivya</t>
+          <t>Sharon</t>
         </is>
       </c>
       <c r="G99" s="10" t="inlineStr">
         <is>
-          <t>Bilal</t>
+          <t>Amit</t>
         </is>
       </c>
       <c r="H99" s="10">
@@ -5885,12 +5886,12 @@
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t>Jithu</t>
+          <t>Neethu</t>
         </is>
       </c>
       <c r="G100" s="10" t="inlineStr">
         <is>
-          <t>Bilsy</t>
+          <t>Vidhu</t>
         </is>
       </c>
       <c r="H100" s="10">
@@ -5924,12 +5925,12 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t>Nivya Peter</t>
+          <t>Nivya Mathew</t>
         </is>
       </c>
       <c r="G101" s="10" t="inlineStr">
         <is>
-          <t>Nikitha</t>
+          <t>Bilal</t>
         </is>
       </c>
       <c r="H101" s="10">
@@ -5943,7 +5944,7 @@
       </c>
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t>Team 2 – Jeem Boom Baa</t>
+          <t>Team 1 – Rajarajeshwari United</t>
         </is>
       </c>
       <c r="C102" s="10" t="inlineStr">
@@ -5963,12 +5964,12 @@
       </c>
       <c r="F102" s="10" t="inlineStr">
         <is>
-          <t>Gokul</t>
+          <t>Jithu</t>
         </is>
       </c>
       <c r="G102" s="10" t="inlineStr">
         <is>
-          <t>Anurag</t>
+          <t>Bilsy</t>
         </is>
       </c>
       <c r="H102" s="10">
@@ -5982,7 +5983,7 @@
       </c>
       <c r="B103" s="10" t="inlineStr">
         <is>
-          <t>Team 2 – Jeem Boom Baa</t>
+          <t>Team 1 – Rajarajeshwari United</t>
         </is>
       </c>
       <c r="C103" s="10" t="inlineStr">
@@ -6002,12 +6003,12 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t>Ray</t>
+          <t>Nivya Peter</t>
         </is>
       </c>
       <c r="G103" s="10" t="inlineStr">
         <is>
-          <t>Boban</t>
+          <t>Nikitha</t>
         </is>
       </c>
       <c r="H103" s="10">
@@ -6041,12 +6042,12 @@
       </c>
       <c r="F104" s="10" t="inlineStr">
         <is>
-          <t>Tressy</t>
+          <t>Gokul K R</t>
         </is>
       </c>
       <c r="G104" s="10" t="inlineStr">
         <is>
-          <t>Shijil</t>
+          <t>Anurag</t>
         </is>
       </c>
       <c r="H104" s="10">
@@ -6080,12 +6081,12 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t>Athira</t>
+          <t>Ray</t>
         </is>
       </c>
       <c r="G105" s="10" t="inlineStr">
         <is>
-          <t>Anas</t>
+          <t>Boban Paul</t>
         </is>
       </c>
       <c r="H105" s="10">
@@ -6119,12 +6120,12 @@
       </c>
       <c r="F106" s="10" t="inlineStr">
         <is>
-          <t>Akshay</t>
+          <t>Tressy</t>
         </is>
       </c>
       <c r="G106" s="10" t="inlineStr">
         <is>
-          <t>Gouresh</t>
+          <t>Shijil</t>
         </is>
       </c>
       <c r="H106" s="10">
@@ -6138,7 +6139,7 @@
       </c>
       <c r="B107" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 2 – Jeem Boom Baa</t>
         </is>
       </c>
       <c r="C107" s="10" t="inlineStr">
@@ -6158,12 +6159,12 @@
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
-          <t>Alwin</t>
+          <t>Athira Jayaprasad</t>
         </is>
       </c>
       <c r="G107" s="10" t="inlineStr">
         <is>
-          <t>Nived</t>
+          <t>Anas</t>
         </is>
       </c>
       <c r="H107" s="10">
@@ -6177,7 +6178,7 @@
       </c>
       <c r="B108" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 2 – Jeem Boom Baa</t>
         </is>
       </c>
       <c r="C108" s="10" t="inlineStr">
@@ -6197,12 +6198,12 @@
       </c>
       <c r="F108" s="10" t="inlineStr">
         <is>
-          <t>Ashmil</t>
+          <t>Akshay</t>
         </is>
       </c>
       <c r="G108" s="10" t="inlineStr">
         <is>
-          <t>Prajith</t>
+          <t>Gouresh</t>
         </is>
       </c>
       <c r="H108" s="10">
@@ -6236,12 +6237,12 @@
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
-          <t>Anan</t>
+          <t>Alwin</t>
         </is>
       </c>
       <c r="G109" s="10" t="inlineStr">
         <is>
-          <t>Avani</t>
+          <t>Nived</t>
         </is>
       </c>
       <c r="H109" s="10">
@@ -6275,12 +6276,12 @@
       </c>
       <c r="F110" s="10" t="inlineStr">
         <is>
-          <t>Nandana</t>
+          <t>Ashmil</t>
         </is>
       </c>
       <c r="G110" s="10" t="inlineStr">
         <is>
-          <t>Sona</t>
+          <t>Prajith</t>
         </is>
       </c>
       <c r="H110" s="10">
@@ -6294,7 +6295,7 @@
       </c>
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t>Team 4 – Thoofan</t>
+          <t>Team 3 – Dr. D</t>
         </is>
       </c>
       <c r="C111" s="10" t="inlineStr">
@@ -6314,12 +6315,12 @@
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
-          <t>Rajeesh C V</t>
+          <t>Anan Nasreen</t>
         </is>
       </c>
       <c r="G111" s="10" t="inlineStr">
         <is>
-          <t>Ibrahim</t>
+          <t>Avani</t>
         </is>
       </c>
       <c r="H111" s="10">
@@ -6333,7 +6334,7 @@
       </c>
       <c r="B112" s="10" t="inlineStr">
         <is>
-          <t>Team 4 – Thoofan</t>
+          <t>Team 3 – Dr. D</t>
         </is>
       </c>
       <c r="C112" s="10" t="inlineStr">
@@ -6353,12 +6354,12 @@
       </c>
       <c r="F112" s="10" t="inlineStr">
         <is>
-          <t>Aparna</t>
+          <t>Nandhana Rayaroth</t>
         </is>
       </c>
       <c r="G112" s="10" t="inlineStr">
         <is>
-          <t>Sahil M I</t>
+          <t>Sona</t>
         </is>
       </c>
       <c r="H112" s="10">
@@ -6392,12 +6393,12 @@
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t>Gautham</t>
+          <t>Rajeesh C V</t>
         </is>
       </c>
       <c r="G113" s="10" t="inlineStr">
         <is>
-          <t>Don</t>
+          <t>Ibrahim</t>
         </is>
       </c>
       <c r="H113" s="10">
@@ -6431,12 +6432,12 @@
       </c>
       <c r="F114" s="10" t="inlineStr">
         <is>
-          <t>Deepanjali</t>
+          <t>Aparna</t>
         </is>
       </c>
       <c r="G114" s="10" t="inlineStr">
         <is>
-          <t>Anjana</t>
+          <t>Sahil M I</t>
         </is>
       </c>
       <c r="H114" s="10">
@@ -6470,12 +6471,12 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t>Samin</t>
+          <t>Gautham</t>
         </is>
       </c>
       <c r="G115" s="10" t="inlineStr">
         <is>
-          <t>Nikhil</t>
+          <t>Don</t>
         </is>
       </c>
       <c r="H115" s="10">
@@ -6489,7 +6490,7 @@
       </c>
       <c r="B116" s="10" t="inlineStr">
         <is>
-          <t>Team 5 – Dhurandhar</t>
+          <t>Team 4 – Thoofan</t>
         </is>
       </c>
       <c r="C116" s="10" t="inlineStr">
@@ -6509,12 +6510,12 @@
       </c>
       <c r="F116" s="10" t="inlineStr">
         <is>
-          <t>Sradha Santhosh</t>
+          <t>Deepanjali</t>
         </is>
       </c>
       <c r="G116" s="10" t="inlineStr">
         <is>
-          <t>Nidheesh P V</t>
+          <t>Anjana</t>
         </is>
       </c>
       <c r="H116" s="10">
@@ -6528,7 +6529,7 @@
       </c>
       <c r="B117" s="10" t="inlineStr">
         <is>
-          <t>Team 5 – Dhurandhar</t>
+          <t>Team 4 – Thoofan</t>
         </is>
       </c>
       <c r="C117" s="10" t="inlineStr">
@@ -6548,12 +6549,12 @@
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
-          <t>Abhishek P S</t>
+          <t>Samin</t>
         </is>
       </c>
       <c r="G117" s="10" t="inlineStr">
         <is>
-          <t>Vidhya M Robert</t>
+          <t>Nikhil</t>
         </is>
       </c>
       <c r="H117" s="10">
@@ -6587,12 +6588,12 @@
       </c>
       <c r="F118" s="10" t="inlineStr">
         <is>
-          <t>Sarath Joseph</t>
+          <t>Sradha Santhosh</t>
         </is>
       </c>
       <c r="G118" s="10" t="inlineStr">
         <is>
-          <t>Adhith Vinoj</t>
+          <t>Nidheesh P V</t>
         </is>
       </c>
       <c r="H118" s="10">
@@ -6626,12 +6627,12 @@
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
-          <t>Abhijith K V</t>
+          <t>Abhishek P S</t>
         </is>
       </c>
       <c r="G119" s="10" t="inlineStr">
         <is>
-          <t>Divin</t>
+          <t>Vidhya M Robert</t>
         </is>
       </c>
       <c r="H119" s="10">
@@ -6645,7 +6646,7 @@
       </c>
       <c r="B120" s="10" t="inlineStr">
         <is>
-          <t>Team 6 – Aaram Thamburan</t>
+          <t>Team 5 – Dhurandhar</t>
         </is>
       </c>
       <c r="C120" s="10" t="inlineStr">
@@ -6665,12 +6666,12 @@
       </c>
       <c r="F120" s="10" t="inlineStr">
         <is>
-          <t>Merrin</t>
+          <t>Sarath Joseph</t>
         </is>
       </c>
       <c r="G120" s="10" t="inlineStr">
         <is>
-          <t>Anandhakrishnan</t>
+          <t>Adhith Vinoj</t>
         </is>
       </c>
       <c r="H120" s="10">
@@ -6684,7 +6685,7 @@
       </c>
       <c r="B121" s="10" t="inlineStr">
         <is>
-          <t>Team 6 – Aaram Thamburan</t>
+          <t>Team 5 – Dhurandhar</t>
         </is>
       </c>
       <c r="C121" s="10" t="inlineStr">
@@ -6704,12 +6705,12 @@
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
-          <t>Ansam</t>
+          <t>Abhijith K V</t>
         </is>
       </c>
       <c r="G121" s="10" t="inlineStr">
         <is>
-          <t>Justin</t>
+          <t>Divin</t>
         </is>
       </c>
       <c r="H121" s="10">
@@ -6743,12 +6744,12 @@
       </c>
       <c r="F122" s="10" t="inlineStr">
         <is>
-          <t>Sharan</t>
+          <t>Merrin</t>
         </is>
       </c>
       <c r="G122" s="10" t="inlineStr">
         <is>
-          <t>Musthaq</t>
+          <t>Anandhakrishnan</t>
         </is>
       </c>
       <c r="H122" s="10">
@@ -6782,12 +6783,12 @@
       </c>
       <c r="F123" s="10" t="inlineStr">
         <is>
-          <t>Akhila</t>
+          <t>Ansam</t>
         </is>
       </c>
       <c r="G123" s="10" t="inlineStr">
         <is>
-          <t>Athira</t>
+          <t>Justin</t>
         </is>
       </c>
       <c r="H123" s="10">
@@ -6821,12 +6822,12 @@
       </c>
       <c r="F124" s="10" t="inlineStr">
         <is>
-          <t>Hrishikesh</t>
+          <t>Sharan</t>
         </is>
       </c>
       <c r="G124" s="10" t="inlineStr">
         <is>
-          <t>Jayakrishnan</t>
+          <t>Musthaq</t>
         </is>
       </c>
       <c r="H124" s="10">
@@ -6860,12 +6861,12 @@
       </c>
       <c r="F125" s="10" t="inlineStr">
         <is>
-          <t>Niju</t>
+          <t>Akhila</t>
         </is>
       </c>
       <c r="G125" s="10" t="inlineStr">
         <is>
-          <t>Christo</t>
+          <t>Athira</t>
         </is>
       </c>
       <c r="H125" s="10">
@@ -6879,30 +6880,34 @@
       </c>
       <c r="B126" s="10" t="inlineStr">
         <is>
-          <t>Team 5 – Dhurandhar</t>
+          <t>Team 6 – Aaram Thamburan</t>
         </is>
       </c>
       <c r="C126" s="10" t="inlineStr">
         <is>
-          <t>Chess</t>
+          <t>Carrom</t>
         </is>
       </c>
       <c r="D126" s="10" t="inlineStr">
         <is>
-          <t>Men</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="E126" s="10" t="inlineStr">
         <is>
-          <t>Singles</t>
+          <t>Doubles</t>
         </is>
       </c>
       <c r="F126" s="10" t="inlineStr">
         <is>
-          <t>Nidheesh P V</t>
-        </is>
-      </c>
-      <c r="G126" s="10" t="n"/>
+          <t>Hrishikesh</t>
+        </is>
+      </c>
+      <c r="G126" s="10" t="inlineStr">
+        <is>
+          <t>Jayakrishnan</t>
+        </is>
+      </c>
       <c r="H126" s="10">
         <f>IF(G126="",F126,F126&amp;" &amp; "&amp;G126)</f>
         <v/>
@@ -6914,30 +6919,34 @@
       </c>
       <c r="B127" s="10" t="inlineStr">
         <is>
-          <t>Team 5 – Dhurandhar</t>
+          <t>Team 6 – Aaram Thamburan</t>
         </is>
       </c>
       <c r="C127" s="10" t="inlineStr">
         <is>
-          <t>Chess</t>
+          <t>Carrom</t>
         </is>
       </c>
       <c r="D127" s="10" t="inlineStr">
         <is>
-          <t>Men</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="E127" s="10" t="inlineStr">
         <is>
-          <t>Singles</t>
+          <t>Doubles</t>
         </is>
       </c>
       <c r="F127" s="10" t="inlineStr">
         <is>
-          <t>Akshay A</t>
-        </is>
-      </c>
-      <c r="G127" s="10" t="n"/>
+          <t>Niju</t>
+        </is>
+      </c>
+      <c r="G127" s="10" t="inlineStr">
+        <is>
+          <t>Christo</t>
+        </is>
+      </c>
       <c r="H127" s="10">
         <f>IF(G127="",F127,F127&amp;" &amp; "&amp;G127)</f>
         <v/>
@@ -6969,7 +6978,7 @@
       </c>
       <c r="F128" s="10" t="inlineStr">
         <is>
-          <t>Bhadresh Das</t>
+          <t>Nidheesh P V</t>
         </is>
       </c>
       <c r="G128" s="10" t="n"/>
@@ -7004,7 +7013,7 @@
       </c>
       <c r="F129" s="10" t="inlineStr">
         <is>
-          <t>Abhijith K V</t>
+          <t>Akshay A</t>
         </is>
       </c>
       <c r="G129" s="10" t="n"/>
@@ -7029,7 +7038,7 @@
       </c>
       <c r="D130" s="10" t="inlineStr">
         <is>
-          <t>Women</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="E130" s="10" t="inlineStr">
@@ -7039,7 +7048,7 @@
       </c>
       <c r="F130" s="10" t="inlineStr">
         <is>
-          <t>Sradha Santhosh</t>
+          <t>Bhadresh Das</t>
         </is>
       </c>
       <c r="G130" s="10" t="n"/>
@@ -7064,7 +7073,7 @@
       </c>
       <c r="D131" s="10" t="inlineStr">
         <is>
-          <t>Women</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="E131" s="10" t="inlineStr">
@@ -7074,7 +7083,7 @@
       </c>
       <c r="F131" s="10" t="inlineStr">
         <is>
-          <t>Mary Metilda</t>
+          <t>Abhijith K V</t>
         </is>
       </c>
       <c r="G131" s="10" t="n"/>
@@ -7089,7 +7098,7 @@
       </c>
       <c r="B132" s="10" t="inlineStr">
         <is>
-          <t>Team 1 – Rajarajeshwari United</t>
+          <t>Team 5 – Dhurandhar</t>
         </is>
       </c>
       <c r="C132" s="10" t="inlineStr">
@@ -7099,7 +7108,7 @@
       </c>
       <c r="D132" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="E132" s="10" t="inlineStr">
@@ -7109,7 +7118,7 @@
       </c>
       <c r="F132" s="10" t="inlineStr">
         <is>
-          <t>Solomon</t>
+          <t>Sradha Santhosh</t>
         </is>
       </c>
       <c r="G132" s="10" t="n"/>
@@ -7124,7 +7133,7 @@
       </c>
       <c r="B133" s="10" t="inlineStr">
         <is>
-          <t>Team 1 – Rajarajeshwari United</t>
+          <t>Team 5 – Dhurandhar</t>
         </is>
       </c>
       <c r="C133" s="10" t="inlineStr">
@@ -7134,7 +7143,7 @@
       </c>
       <c r="D133" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="E133" s="10" t="inlineStr">
@@ -7144,7 +7153,7 @@
       </c>
       <c r="F133" s="10" t="inlineStr">
         <is>
-          <t>Nivya</t>
+          <t>Mary Metilda</t>
         </is>
       </c>
       <c r="G133" s="10" t="n"/>
@@ -7179,7 +7188,7 @@
       </c>
       <c r="F134" s="10" t="inlineStr">
         <is>
-          <t>Jithu</t>
+          <t>Solomon</t>
         </is>
       </c>
       <c r="G134" s="10" t="n"/>
@@ -7214,7 +7223,7 @@
       </c>
       <c r="F135" s="10" t="inlineStr">
         <is>
-          <t>Shamil</t>
+          <t>Nivya Mathew</t>
         </is>
       </c>
       <c r="G135" s="10" t="n"/>
@@ -7229,7 +7238,7 @@
       </c>
       <c r="B136" s="10" t="inlineStr">
         <is>
-          <t>Team 2 – Jeem Boom Baa</t>
+          <t>Team 1 – Rajarajeshwari United</t>
         </is>
       </c>
       <c r="C136" s="10" t="inlineStr">
@@ -7249,7 +7258,7 @@
       </c>
       <c r="F136" s="10" t="inlineStr">
         <is>
-          <t>Shijil</t>
+          <t>Jithu</t>
         </is>
       </c>
       <c r="G136" s="10" t="n"/>
@@ -7264,7 +7273,7 @@
       </c>
       <c r="B137" s="10" t="inlineStr">
         <is>
-          <t>Team 2 – Jeem Boom Baa</t>
+          <t>Team 1 – Rajarajeshwari United</t>
         </is>
       </c>
       <c r="C137" s="10" t="inlineStr">
@@ -7284,7 +7293,7 @@
       </c>
       <c r="F137" s="10" t="inlineStr">
         <is>
-          <t>Bonny</t>
+          <t>Shamil</t>
         </is>
       </c>
       <c r="G137" s="10" t="n"/>
@@ -7319,7 +7328,7 @@
       </c>
       <c r="F138" s="10" t="inlineStr">
         <is>
-          <t>Sravan</t>
+          <t>Shijil</t>
         </is>
       </c>
       <c r="G138" s="10" t="n"/>
@@ -7354,7 +7363,7 @@
       </c>
       <c r="F139" s="10" t="inlineStr">
         <is>
-          <t>Anurag</t>
+          <t>Bonny</t>
         </is>
       </c>
       <c r="G139" s="10" t="n"/>
@@ -7389,7 +7398,7 @@
       </c>
       <c r="F140" s="10" t="inlineStr">
         <is>
-          <t>Renson</t>
+          <t>Sravan</t>
         </is>
       </c>
       <c r="G140" s="10" t="n"/>
@@ -7424,7 +7433,7 @@
       </c>
       <c r="F141" s="10" t="inlineStr">
         <is>
-          <t>Sainal</t>
+          <t>Anurag</t>
         </is>
       </c>
       <c r="G141" s="10" t="n"/>
@@ -7459,7 +7468,7 @@
       </c>
       <c r="F142" s="10" t="inlineStr">
         <is>
-          <t>Gokul</t>
+          <t>Renson</t>
         </is>
       </c>
       <c r="G142" s="10" t="n"/>
@@ -7494,7 +7503,7 @@
       </c>
       <c r="F143" s="10" t="inlineStr">
         <is>
-          <t>Ray</t>
+          <t>Sainal</t>
         </is>
       </c>
       <c r="G143" s="10" t="n"/>
@@ -7509,7 +7518,7 @@
       </c>
       <c r="B144" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 2 – Jeem Boom Baa</t>
         </is>
       </c>
       <c r="C144" s="10" t="inlineStr">
@@ -7529,7 +7538,7 @@
       </c>
       <c r="F144" s="10" t="inlineStr">
         <is>
-          <t>Ashmil</t>
+          <t>Gokul K R</t>
         </is>
       </c>
       <c r="G144" s="10" t="n"/>
@@ -7544,7 +7553,7 @@
       </c>
       <c r="B145" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 2 – Jeem Boom Baa</t>
         </is>
       </c>
       <c r="C145" s="10" t="inlineStr">
@@ -7564,7 +7573,7 @@
       </c>
       <c r="F145" s="10" t="inlineStr">
         <is>
-          <t>Nived</t>
+          <t>Ray</t>
         </is>
       </c>
       <c r="G145" s="10" t="n"/>
@@ -7599,7 +7608,7 @@
       </c>
       <c r="F146" s="10" t="inlineStr">
         <is>
-          <t>Anjaly</t>
+          <t>Ashmil</t>
         </is>
       </c>
       <c r="G146" s="10" t="n"/>
@@ -7634,7 +7643,7 @@
       </c>
       <c r="F147" s="10" t="inlineStr">
         <is>
-          <t>Anan</t>
+          <t>Nived</t>
         </is>
       </c>
       <c r="G147" s="10" t="n"/>
@@ -7649,7 +7658,7 @@
       </c>
       <c r="B148" s="10" t="inlineStr">
         <is>
-          <t>Team 4 – Thoofan</t>
+          <t>Team 3 – Dr. D</t>
         </is>
       </c>
       <c r="C148" s="10" t="inlineStr">
@@ -7669,7 +7678,7 @@
       </c>
       <c r="F148" s="10" t="inlineStr">
         <is>
-          <t>Samin</t>
+          <t>Anjaly C Prakash</t>
         </is>
       </c>
       <c r="G148" s="10" t="n"/>
@@ -7684,7 +7693,7 @@
       </c>
       <c r="B149" s="10" t="inlineStr">
         <is>
-          <t>Team 4 – Thoofan</t>
+          <t>Team 3 – Dr. D</t>
         </is>
       </c>
       <c r="C149" s="10" t="inlineStr">
@@ -7704,7 +7713,7 @@
       </c>
       <c r="F149" s="10" t="inlineStr">
         <is>
-          <t>Rajeesh C V</t>
+          <t>Anan Nasreen</t>
         </is>
       </c>
       <c r="G149" s="10" t="n"/>
@@ -7739,7 +7748,7 @@
       </c>
       <c r="F150" s="10" t="inlineStr">
         <is>
-          <t>Gautham</t>
+          <t>Samin</t>
         </is>
       </c>
       <c r="G150" s="10" t="n"/>
@@ -7774,7 +7783,7 @@
       </c>
       <c r="F151" s="10" t="inlineStr">
         <is>
-          <t>AnnMary</t>
+          <t>Rajeesh C V</t>
         </is>
       </c>
       <c r="G151" s="10" t="n"/>
@@ -7789,7 +7798,7 @@
       </c>
       <c r="B152" s="10" t="inlineStr">
         <is>
-          <t>Team 6 – Aaram Thamburan</t>
+          <t>Team 4 – Thoofan</t>
         </is>
       </c>
       <c r="C152" s="10" t="inlineStr">
@@ -7809,7 +7818,7 @@
       </c>
       <c r="F152" s="10" t="inlineStr">
         <is>
-          <t>Akshaya</t>
+          <t>Gautham</t>
         </is>
       </c>
       <c r="G152" s="10" t="n"/>
@@ -7824,7 +7833,7 @@
       </c>
       <c r="B153" s="10" t="inlineStr">
         <is>
-          <t>Team 6 – Aaram Thamburan</t>
+          <t>Team 4 – Thoofan</t>
         </is>
       </c>
       <c r="C153" s="10" t="inlineStr">
@@ -7844,7 +7853,7 @@
       </c>
       <c r="F153" s="10" t="inlineStr">
         <is>
-          <t>Merrin</t>
+          <t>AnnMary</t>
         </is>
       </c>
       <c r="G153" s="10" t="n"/>
@@ -7879,7 +7888,7 @@
       </c>
       <c r="F154" s="10" t="inlineStr">
         <is>
-          <t>Benison</t>
+          <t>Akshaya</t>
         </is>
       </c>
       <c r="G154" s="10" t="n"/>
@@ -7914,7 +7923,7 @@
       </c>
       <c r="F155" s="10" t="inlineStr">
         <is>
-          <t>Hrishikesh</t>
+          <t>Merrin</t>
         </is>
       </c>
       <c r="G155" s="10" t="n"/>
@@ -7949,7 +7958,7 @@
       </c>
       <c r="F156" s="10" t="inlineStr">
         <is>
-          <t>Neha</t>
+          <t>Benison</t>
         </is>
       </c>
       <c r="G156" s="10" t="n"/>
@@ -7958,8 +7967,76 @@
         <v/>
       </c>
     </row>
-    <row r="157" ht="15.75" customHeight="1" s="15"/>
-    <row r="158" ht="15.75" customHeight="1" s="15"/>
+    <row r="157" ht="15.75" customHeight="1" s="15">
+      <c r="A157" s="10" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" s="10" t="inlineStr">
+        <is>
+          <t>Team 6 – Aaram Thamburan</t>
+        </is>
+      </c>
+      <c r="C157" s="10" t="inlineStr">
+        <is>
+          <t>Chess</t>
+        </is>
+      </c>
+      <c r="D157" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E157" s="10" t="inlineStr">
+        <is>
+          <t>Singles</t>
+        </is>
+      </c>
+      <c r="F157" s="10" t="inlineStr">
+        <is>
+          <t>Hrishikesh</t>
+        </is>
+      </c>
+      <c r="G157" s="10" t="n"/>
+      <c r="H157" s="10">
+        <f>IF(G157="",F157,F157&amp;" &amp; "&amp;G157)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="158" ht="15.75" customHeight="1" s="15">
+      <c r="A158" s="10" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" s="10" t="inlineStr">
+        <is>
+          <t>Team 6 – Aaram Thamburan</t>
+        </is>
+      </c>
+      <c r="C158" s="10" t="inlineStr">
+        <is>
+          <t>Chess</t>
+        </is>
+      </c>
+      <c r="D158" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E158" s="10" t="inlineStr">
+        <is>
+          <t>Singles</t>
+        </is>
+      </c>
+      <c r="F158" s="10" t="inlineStr">
+        <is>
+          <t>Neha</t>
+        </is>
+      </c>
+      <c r="G158" s="10" t="n"/>
+      <c r="H158" s="10">
+        <f>IF(G158="",F158,F158&amp;" &amp; "&amp;G158)</f>
+        <v/>
+      </c>
+    </row>
     <row r="159" ht="15.75" customHeight="1" s="15"/>
     <row r="160" ht="15.75" customHeight="1" s="15"/>
     <row r="161" ht="15.75" customHeight="1" s="15"/>
@@ -8818,7 +8895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="5" customWidth="1" style="15" min="1" max="1"/>
@@ -8914,7 +8991,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Gokul</t>
+          <t>Amal Jose</t>
         </is>
       </c>
       <c r="D7" s="6" t="n"/>
@@ -8931,7 +9008,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Amal</t>
+          <t>Gokul K R</t>
         </is>
       </c>
       <c r="D8" s="6" t="n"/>
@@ -8948,7 +9025,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Kevin</t>
+          <t>Kevin Raj</t>
         </is>
       </c>
       <c r="D9" s="6" t="n"/>
@@ -8965,7 +9042,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Adwaith</t>
+          <t>Adwaith Narayanan</t>
         </is>
       </c>
       <c r="D10" s="6" t="n"/>
@@ -8982,7 +9059,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Sahil M I</t>
+          <t>Anandhan Sreekumar</t>
         </is>
       </c>
       <c r="D11" s="6" t="n"/>
@@ -8999,7 +9076,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Rajeesh C V</t>
+          <t>Soorya Thejas</t>
         </is>
       </c>
       <c r="D12" s="6" t="n"/>
@@ -9016,7 +9093,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Adhith Vinoj</t>
+          <t>Nidheesh P V</t>
         </is>
       </c>
       <c r="D13" s="6" t="n"/>
@@ -9033,7 +9110,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Nidheesh P V</t>
+          <t>Adhith Vinoj</t>
         </is>
       </c>
       <c r="D14" s="6" t="n"/>
@@ -9050,7 +9127,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Joel</t>
+          <t>Joel Paul</t>
         </is>
       </c>
       <c r="D15" s="6" t="n"/>
@@ -9067,12 +9144,13 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Jayesh</t>
+          <t>Musthaq</t>
         </is>
       </c>
       <c r="D16" s="6" t="n"/>
       <c r="E16" s="7" t="n"/>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
@@ -9135,7 +9213,7 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Nivya</t>
+          <t>Nivya Mathew</t>
         </is>
       </c>
       <c r="D21" s="6" t="n"/>
@@ -9152,7 +9230,7 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Tressy</t>
+          <t>Anima V Shaji</t>
         </is>
       </c>
       <c r="D22" s="6" t="n"/>
@@ -9169,7 +9247,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Anima</t>
+          <t>Tressy</t>
         </is>
       </c>
       <c r="D23" s="6" t="n"/>
@@ -9186,7 +9264,7 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Anjaly</t>
+          <t>Anjaly C Prakash</t>
         </is>
       </c>
       <c r="D24" s="6" t="n"/>
@@ -9203,7 +9281,7 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Fadwah</t>
+          <t>Neha Abdul Majeed</t>
         </is>
       </c>
       <c r="D25" s="6" t="n"/>
@@ -9305,7 +9383,7 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Akshaya</t>
+          <t>Ashna</t>
         </is>
       </c>
       <c r="D31" s="6" t="n"/>
@@ -9387,7 +9465,7 @@
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Jithu</t>
+          <t>Shamil</t>
         </is>
       </c>
       <c r="E36" s="7" t="n"/>
@@ -9403,12 +9481,12 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Gokul</t>
+          <t>Amal Jose</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Amal</t>
+          <t>Gokul K R</t>
         </is>
       </c>
       <c r="E37" s="7" t="n"/>
@@ -9429,7 +9507,7 @@
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>Sravan</t>
+          <t>Boban Paul</t>
         </is>
       </c>
       <c r="E38" s="7" t="n"/>
@@ -9445,12 +9523,12 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Ashmil</t>
+          <t>Kevin Raj</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Jerishab</t>
+          <t>Adwaith Narayanan</t>
         </is>
       </c>
       <c r="E39" s="7" t="n"/>
@@ -9466,12 +9544,12 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Rithik</t>
+          <t>Rithik P Vijay</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>Jerin</t>
+          <t>Jerin Wilson</t>
         </is>
       </c>
       <c r="E40" s="7" t="n"/>
@@ -9487,12 +9565,12 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Sahil M I</t>
+          <t>Rajeesh C V</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>Rajeesh C V</t>
+          <t>Akhil P Jose</t>
         </is>
       </c>
       <c r="E41" s="7" t="n"/>
@@ -9508,7 +9586,7 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Don</t>
+          <t>Sahil M I</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
@@ -9545,17 +9623,17 @@
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>Team 6 – Aaram Thamburan</t>
+          <t>Team 5 – Dhurandhar</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Joel</t>
+          <t>Abhijith K V</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>Jayesh</t>
+          <t>Akshay A</t>
         </is>
       </c>
       <c r="E44" s="7" t="n"/>
@@ -9571,7 +9649,7 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Sharan</t>
+          <t>Joel Paul</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
@@ -9581,69 +9659,69 @@
       </c>
       <c r="E45" s="7" t="n"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" s="15"/>
-    <row r="47" ht="15.75" customHeight="1" s="15">
-      <c r="A47" s="2" t="inlineStr">
+    <row r="46" ht="15.75" customHeight="1" s="15">
+      <c r="A46" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>Team 6 – Aaram Thamburan</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Jayesh</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>Ansam</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="n"/>
+    </row>
+    <row r="47" ht="15.75" customHeight="1" s="15"/>
+    <row r="48" ht="15.75" customHeight="1" s="15">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>Women’s Doubles</t>
         </is>
       </c>
-      <c r="B47" s="3" t="n"/>
-      <c r="C47" s="3" t="n"/>
-      <c r="D47" s="3" t="n"/>
-      <c r="E47" s="3" t="n"/>
-    </row>
-    <row r="48" ht="15.75" customHeight="1" s="15">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="B48" s="3" t="n"/>
+      <c r="C48" s="3" t="n"/>
+      <c r="D48" s="3" t="n"/>
+      <c r="E48" s="3" t="n"/>
+    </row>
+    <row r="49" ht="15.75" customHeight="1" s="15">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B49" s="8" t="inlineStr">
         <is>
           <t>Team</t>
         </is>
       </c>
-      <c r="C48" s="8" t="inlineStr">
+      <c r="C49" s="8" t="inlineStr">
         <is>
           <t>Player 1</t>
         </is>
       </c>
-      <c r="D48" s="8" t="inlineStr">
+      <c r="D49" s="8" t="inlineStr">
         <is>
           <t>Player 2</t>
         </is>
       </c>
-      <c r="E48" s="8" t="inlineStr">
+      <c r="E49" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-    </row>
-    <row r="49" ht="15.75" customHeight="1" s="15">
-      <c r="A49" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>Team 1 – Rajarajeshwari United</t>
-        </is>
-      </c>
-      <c r="C49" s="6" t="inlineStr">
-        <is>
-          <t>Neethu</t>
-        </is>
-      </c>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>Nivya Mathew</t>
-        </is>
-      </c>
-      <c r="E49" s="7" t="n"/>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="15">
       <c r="A50" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
@@ -9652,40 +9730,40 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Nivya Peter</t>
+          <t>Neethu</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>Bilsy</t>
+          <t>Nivya Mathew</t>
         </is>
       </c>
       <c r="E50" s="7" t="n"/>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="15">
       <c r="A51" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>Team 2 – Jeem Boom Baa</t>
+          <t>Team 1 – Rajarajeshwari United</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Tressy</t>
+          <t>Shinu</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Anima</t>
+          <t>Bilsy</t>
         </is>
       </c>
       <c r="E51" s="7" t="n"/>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="15">
       <c r="A52" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
@@ -9694,40 +9772,40 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Surya</t>
+          <t>Josna Mathew</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>Josna</t>
+          <t>Athira Jayaprasad</t>
         </is>
       </c>
       <c r="E52" s="7" t="n"/>
     </row>
     <row r="53" ht="15.75" customHeight="1" s="15">
       <c r="A53" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 2 – Jeem Boom Baa</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>Anjaly</t>
+          <t>Anima V Shaji</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Fadwah</t>
+          <t>Tressy</t>
         </is>
       </c>
       <c r="E53" s="7" t="n"/>
     </row>
     <row r="54" ht="15.75" customHeight="1" s="15">
       <c r="A54" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
@@ -9736,40 +9814,40 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>Neha</t>
+          <t>Anjaly C Prakash</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Nandana</t>
+          <t>Anan Nasreen</t>
         </is>
       </c>
       <c r="E54" s="7" t="n"/>
     </row>
     <row r="55" ht="15.75" customHeight="1" s="15">
       <c r="A55" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>Team 4 – Thoofan</t>
+          <t>Team 3 – Dr. D</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>Manjusha</t>
+          <t>Neha Abdul Majeed</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>AnnMary</t>
+          <t>Nandhana Rayaroth</t>
         </is>
       </c>
       <c r="E55" s="7" t="n"/>
     </row>
     <row r="56" ht="15.75" customHeight="1" s="15">
       <c r="A56" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
@@ -9778,85 +9856,121 @@
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>Aparna</t>
+          <t>Manjusha</t>
         </is>
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>Gayathri</t>
+          <t>AnnMary</t>
         </is>
       </c>
       <c r="E56" s="7" t="n"/>
     </row>
     <row r="57" ht="15.75" customHeight="1" s="15">
       <c r="A57" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>Team 5 – Dhurandhar</t>
+          <t>Team 4 – Thoofan</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>Sradha Santhosh</t>
+          <t>Aparna</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>Vidhya M Robert</t>
+          <t>Gayathri</t>
         </is>
       </c>
       <c r="E57" s="7" t="n"/>
     </row>
     <row r="58" ht="15.75" customHeight="1" s="15">
       <c r="A58" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>Team 6 – Aaram Thamburan</t>
+          <t>Team 5 – Dhurandhar</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>Merrin</t>
+          <t>Riya Fathima</t>
         </is>
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>Akshaya</t>
+          <t>Ameesha T</t>
         </is>
       </c>
       <c r="E58" s="7" t="n"/>
     </row>
     <row r="59" ht="15.75" customHeight="1" s="15">
       <c r="A59" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>Team 5 – Dhurandhar</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>Sradha Santhosh</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>Vidhya M Robert</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="n"/>
+    </row>
+    <row r="60" ht="15.75" customHeight="1" s="15">
+      <c r="A60" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B59" s="6" t="inlineStr">
+      <c r="B60" s="6" t="inlineStr">
         <is>
           <t>Team 6 – Aaram Thamburan</t>
         </is>
       </c>
-      <c r="C59" s="6" t="inlineStr">
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>Merrin</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
         <is>
           <t>Ashna</t>
         </is>
       </c>
-      <c r="D59" s="6" t="inlineStr">
-        <is>
-          <t>Akhila / Athira</t>
-        </is>
-      </c>
-      <c r="E59" s="7" t="inlineStr">
-        <is>
-          <t>Partner not final: Akhila OR Athira</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="15.75" customHeight="1" s="15"/>
-    <row r="61" ht="15.75" customHeight="1" s="15"/>
+      <c r="E60" s="7" t="n"/>
+    </row>
+    <row r="61" ht="15.75" customHeight="1" s="15">
+      <c r="A61" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>Team 6 – Aaram Thamburan</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>Akshaya</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>Athira</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="n"/>
+    </row>
     <row r="62" ht="15.75" customHeight="1" s="15"/>
     <row r="63" ht="15.75" customHeight="1" s="15"/>
     <row r="64" ht="15.75" customHeight="1" s="15"/>
@@ -10825,6 +10939,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -11010,7 +11125,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Rithik</t>
+          <t>Rithik P Vijay</t>
         </is>
       </c>
       <c r="D13" s="6" t="n"/>
@@ -11044,7 +11159,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Adwaith</t>
+          <t>Adwaith Narayanan</t>
         </is>
       </c>
       <c r="D15" s="6" t="n"/>
@@ -11112,7 +11227,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Suryathejas</t>
+          <t>Soorya Thejas</t>
         </is>
       </c>
       <c r="D19" s="6" t="n"/>
@@ -11321,7 +11436,7 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Anan</t>
+          <t>Anan Nasreen</t>
         </is>
       </c>
       <c r="D32" s="6" t="n"/>
@@ -11567,7 +11682,7 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Adwaith</t>
+          <t>Adwaith Narayanan</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -11609,7 +11724,7 @@
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Rithik</t>
+          <t>Rithik P Vijay</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
@@ -11635,7 +11750,7 @@
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>Suryathejas</t>
+          <t>Soorya Thejas</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
@@ -12820,6 +12935,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -12953,7 +13069,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Nivya</t>
+          <t>Nivya Mathew</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -13016,7 +13132,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Gokul</t>
+          <t>Gokul K R</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -13042,7 +13158,7 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Boban</t>
+          <t>Boban Paul</t>
         </is>
       </c>
       <c r="E13" s="7" t="n"/>
@@ -13079,7 +13195,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Athira</t>
+          <t>Athira Jayaprasad</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -13167,7 +13283,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Anan</t>
+          <t>Anan Nasreen</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -13188,7 +13304,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Nandana</t>
+          <t>Nandhana Rayaroth</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -14511,6 +14627,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -14613,6 +14730,7 @@
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="7" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
@@ -14681,6 +14799,7 @@
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="7" t="n"/>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
@@ -14743,7 +14862,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Nivya</t>
+          <t>Nivya Mathew</t>
         </is>
       </c>
       <c r="D18" s="6" t="n"/>
@@ -14896,7 +15015,7 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Gokul</t>
+          <t>Gokul K R</t>
         </is>
       </c>
       <c r="D27" s="6" t="n"/>
@@ -14964,7 +15083,7 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Anjaly</t>
+          <t>Anjaly C Prakash</t>
         </is>
       </c>
       <c r="D31" s="6" t="n"/>
@@ -14981,7 +15100,7 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Anan</t>
+          <t>Anan Nasreen</t>
         </is>
       </c>
       <c r="D32" s="6" t="n"/>

</xml_diff>

<commit_message>
Rename Dr. D to Dr. Dashamoolam and sync Dhurandhar badminton changes
Fallback data now matches the Google Sheet:
- Team 3 is renamed Dr. Dashamoolam (Standings, Cricket and Football pools,
  Participants workbook)
- Dhurandhar badminton swaps: Ameesha T (WS), Akshay A (MS),
  Sradha Santhosh & Aryamol (WD), Nidheesh P V & Gowtham A P (MD)
- BWS-R1-01 and BWD-R1-03 swap slots (11:12 Court 1 / 11:30 Court 2) so
  Ameesha T gets her rest between singles and doubles

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XgUQLqsKTbyKtnK2HPdyHV
</commit_message>
<xml_diff>
--- a/data/Vonnue_Cup_Participants.xlsx
+++ b/data/Vonnue_Cup_Participants.xlsx
@@ -564,7 +564,7 @@
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
@@ -1186,7 +1186,7 @@
         <v>18</v>
       </c>
       <c r="H18" s="14" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I18" s="14" t="n">
         <v>18</v>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>Adhith Vinoj</t>
+          <t>Akshay A</t>
         </is>
       </c>
       <c r="G11" s="10" t="n"/>
@@ -2820,7 +2820,7 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
@@ -2855,7 +2855,7 @@
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
@@ -3015,7 +3015,7 @@
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>Vidhya M Robert</t>
+          <t>Ameesha T</t>
         </is>
       </c>
       <c r="G23" s="10" t="n"/>
@@ -3256,7 +3256,7 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
@@ -3437,7 +3437,7 @@
       </c>
       <c r="G34" s="10" t="inlineStr">
         <is>
-          <t>Adhith Vinoj</t>
+          <t>Gowtham A P</t>
         </is>
       </c>
       <c r="H34" s="10">
@@ -3724,7 +3724,7 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
@@ -3944,7 +3944,7 @@
       </c>
       <c r="G47" s="10" t="inlineStr">
         <is>
-          <t>Vidhya M Robert</t>
+          <t>Aryamol</t>
         </is>
       </c>
       <c r="H47" s="10">
@@ -4316,7 +4316,7 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
@@ -4351,7 +4351,7 @@
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
@@ -4386,7 +4386,7 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
@@ -4421,7 +4421,7 @@
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
@@ -4456,7 +4456,7 @@
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C74" s="10" t="inlineStr">
@@ -5281,7 +5281,7 @@
       </c>
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C85" s="10" t="inlineStr">
@@ -5320,7 +5320,7 @@
       </c>
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
@@ -5359,7 +5359,7 @@
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C87" s="10" t="inlineStr">
@@ -6217,7 +6217,7 @@
       </c>
       <c r="B109" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C109" s="10" t="inlineStr">
@@ -6256,7 +6256,7 @@
       </c>
       <c r="B110" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C110" s="10" t="inlineStr">
@@ -6295,7 +6295,7 @@
       </c>
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C111" s="10" t="inlineStr">
@@ -6334,7 +6334,7 @@
       </c>
       <c r="B112" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C112" s="10" t="inlineStr">
@@ -7588,7 +7588,7 @@
       </c>
       <c r="B146" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C146" s="10" t="inlineStr">
@@ -7623,7 +7623,7 @@
       </c>
       <c r="B147" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C147" s="10" t="inlineStr">
@@ -7658,7 +7658,7 @@
       </c>
       <c r="B148" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C148" s="10" t="inlineStr">
@@ -7693,7 +7693,7 @@
       </c>
       <c r="B149" s="10" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C149" s="10" t="inlineStr">
@@ -8912,6 +8912,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -9020,7 +9021,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -9037,7 +9038,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -9110,7 +9111,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Adhith Vinoj</t>
+          <t>Akshay A</t>
         </is>
       </c>
       <c r="D14" s="6" t="n"/>
@@ -9259,7 +9260,7 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -9276,7 +9277,7 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -9349,7 +9350,7 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Vidhya M Robert</t>
+          <t>Ameesha T</t>
         </is>
       </c>
       <c r="D29" s="6" t="n"/>
@@ -9518,7 +9519,7 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
@@ -9539,7 +9540,7 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -9612,7 +9613,7 @@
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>Adhith Vinoj</t>
+          <t>Gowtham A P</t>
         </is>
       </c>
       <c r="E43" s="7" t="n"/>
@@ -9809,7 +9810,7 @@
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -9830,7 +9831,7 @@
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -9924,7 +9925,7 @@
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Vidhya M Robert</t>
+          <t>Aryamol</t>
         </is>
       </c>
       <c r="E59" s="7" t="n"/>
@@ -11120,7 +11121,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -11137,7 +11138,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -11154,7 +11155,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -11171,7 +11172,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -11188,7 +11189,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -11431,7 +11432,7 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -11677,7 +11678,7 @@
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -11698,7 +11699,7 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -11719,7 +11720,7 @@
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -13236,7 +13237,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -13257,7 +13258,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -13278,7 +13279,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -13299,7 +13300,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -15044,7 +15045,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -15061,7 +15062,7 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -15078,7 +15079,7 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -15095,7 +15096,7 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Team 3 – Dr. D</t>
+          <t>Team 3 – Dr. Dashamoolam</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">

</xml_diff>